<commit_message>
Entrevistas E1-E4 en las necesidades y sin comentarios en Asana
- Entrevistas a estudiantes de Sebastián (F-07) como FOOD4ALL_entrevistas_estudiantes.md y anexo C2 del documento final.
- Estados provisionales: N-PLA-01, N-PLA-02, N-CAR-01, N-CAD-01 y N-CAT-01 pasan a Indicio; N-IA-01 queda No confirmada (apartado 5.1 de FOOD4ALL_necesidades.md). Faltan las entrevistas del resto del equipo.
- actualizar_asana.js ya no publica comentarios (se quita --comentar-criba).
- Registro de prompts del 22 y 23/10.
</commit_message>
<xml_diff>
--- a/docs/requisitos/FOOD4ALL_requisitos_benchmark.xlsx
+++ b/docs/requisitos/FOOD4ALL_requisitos_benchmark.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14618" uniqueCount="2788">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14618" uniqueCount="2790">
   <si>
     <t>FOOD4ALL · Catálogo de requisitos con benchmark</t>
   </si>
@@ -7031,7 +7031,10 @@
     <t>Usuario</t>
   </si>
   <si>
-    <t>F-01, F-02</t>
+    <t>Indicio</t>
+  </si>
+  <si>
+    <t>F-01, F-02, F-07 (E3, E4)</t>
   </si>
   <si>
     <t>N-01</t>
@@ -7040,10 +7043,10 @@
     <t>N-03, N-04, N-05</t>
   </si>
   <si>
-    <t>F-01</t>
-  </si>
-  <si>
-    <t>F-04, F-10</t>
+    <t>F-01, F-07 (E4; E1 comparativo)</t>
+  </si>
+  <si>
+    <t>F-04, F-10, F-07 (E4; E3 en contra del producto, no de la necesidad)</t>
   </si>
   <si>
     <t>N-02</t>
@@ -7058,7 +7061,7 @@
     <t>N-10</t>
   </si>
   <si>
-    <t>F-01, F-03</t>
+    <t>F-01, F-03, F-07 (E3, E4)</t>
   </si>
   <si>
     <t>N-08</t>
@@ -7067,7 +7070,10 @@
     <t>N-06, N-07</t>
   </si>
   <si>
-    <t>F-02</t>
+    <t>No confirmada</t>
+  </si>
+  <si>
+    <t>F-02, F-07 (en contra: E3, E4)</t>
   </si>
   <si>
     <t>N-01 (parte)</t>
@@ -7088,7 +7094,7 @@
     <t>—</t>
   </si>
   <si>
-    <t>F-03 (Reglamento 178/2002), F-04</t>
+    <t>F-03 (Reglamento 178/2002), F-04, F-07 (E4; E1 y E2 comparativos)</t>
   </si>
   <si>
     <t>N-04 y N-05 (parte)</t>
@@ -50614,16 +50620,16 @@
         <v>2310</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>921</v>
+        <v>2311</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>2311</v>
+        <v>2312</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>2312</v>
+        <v>2313</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>2313</v>
+        <v>2314</v>
       </c>
       <c r="I2" s="2">
         <v>21</v>
@@ -50646,16 +50652,16 @@
         <v>2310</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>921</v>
+        <v>2311</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>2314</v>
+        <v>2315</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>2312</v>
+        <v>2313</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>2312</v>
+        <v>2313</v>
       </c>
       <c r="I3" s="2">
         <v>19</v>
@@ -50678,16 +50684,16 @@
         <v>2310</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>921</v>
+        <v>2311</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>2315</v>
+        <v>2316</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>2316</v>
+        <v>2317</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>2317</v>
+        <v>2318</v>
       </c>
       <c r="I4" s="2">
         <v>162</v>
@@ -50713,13 +50719,13 @@
         <v>921</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>2318</v>
+        <v>2319</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>2316</v>
+        <v>2317</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>2319</v>
+        <v>2320</v>
       </c>
       <c r="I5" s="2">
         <v>33</v>
@@ -50742,16 +50748,16 @@
         <v>2310</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>921</v>
+        <v>2311</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>2320</v>
+        <v>2321</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>2321</v>
+        <v>2322</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>2322</v>
+        <v>2323</v>
       </c>
       <c r="I6" s="2">
         <v>8</v>
@@ -50774,16 +50780,16 @@
         <v>2310</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>921</v>
+        <v>2324</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>2323</v>
+        <v>2325</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>2324</v>
+        <v>2326</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>2325</v>
+        <v>2327</v>
       </c>
       <c r="I7" s="2">
         <v>10</v>
@@ -50803,19 +50809,19 @@
         <v>2309</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>2327</v>
+        <v>2329</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>2328</v>
+        <v>2330</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="I8" s="2">
         <v>11</v>
@@ -50838,16 +50844,16 @@
         <v>2310</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>921</v>
+        <v>2311</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>2330</v>
+        <v>2332</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>2331</v>
+        <v>2333</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="I9" s="2">
         <v>36</v>
@@ -50867,19 +50873,19 @@
         <v>2309</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>2333</v>
+        <v>2335</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>2334</v>
+        <v>2336</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="I10" s="2">
         <v>14</v>
@@ -50899,19 +50905,19 @@
         <v>2309</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>2335</v>
+        <v>2337</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>2328</v>
+        <v>2330</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="I11" s="2">
         <v>35</v>
@@ -50928,22 +50934,22 @@
         <v>115</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>2336</v>
+        <v>2338</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>2337</v>
+        <v>2339</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>2328</v>
+        <v>2330</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="I12" s="2">
         <v>61</v>
@@ -50969,13 +50975,13 @@
         <v>921</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>2338</v>
+        <v>2340</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>2339</v>
+        <v>2341</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="I13" s="2">
         <v>34</v>
@@ -50992,7 +50998,7 @@
         <v>405</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>2340</v>
+        <v>2342</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>2310</v>
@@ -51001,13 +51007,13 @@
         <v>921</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>2341</v>
+        <v>2343</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>2342</v>
+        <v>2344</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>2343</v>
+        <v>2345</v>
       </c>
       <c r="I14" s="2">
         <v>15</v>
@@ -51024,7 +51030,7 @@
         <v>316</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>2340</v>
+        <v>2342</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>2310</v>
@@ -51033,13 +51039,13 @@
         <v>921</v>
       </c>
       <c r="F15" s="2" t="s">
+        <v>2346</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>2344</v>
       </c>
-      <c r="G15" s="2" t="s">
-        <v>2342</v>
-      </c>
       <c r="H15" s="2" t="s">
-        <v>2345</v>
+        <v>2347</v>
       </c>
       <c r="I15" s="2">
         <v>16</v>
@@ -51056,7 +51062,7 @@
         <v>837</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>2340</v>
+        <v>2342</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>2310</v>
@@ -51065,13 +51071,13 @@
         <v>921</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>2346</v>
+        <v>2348</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>2347</v>
+        <v>2349</v>
       </c>
       <c r="I16" s="2">
         <v>1</v>
@@ -51088,7 +51094,7 @@
         <v>1155</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>2340</v>
+        <v>2342</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>2310</v>
@@ -51097,13 +51103,13 @@
         <v>921</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>2348</v>
+        <v>2350</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>2349</v>
+        <v>2351</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>2350</v>
+        <v>2352</v>
       </c>
       <c r="I17" s="2">
         <v>13</v>
@@ -51120,7 +51126,7 @@
         <v>418</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>2340</v>
+        <v>2342</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>2310</v>
@@ -51129,13 +51135,13 @@
         <v>921</v>
       </c>
       <c r="F18" s="2" t="s">
+        <v>2353</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>2351</v>
       </c>
-      <c r="G18" s="2" t="s">
-        <v>2349</v>
-      </c>
       <c r="H18" s="2" t="s">
-        <v>2352</v>
+        <v>2354</v>
       </c>
       <c r="I18" s="2">
         <v>11</v>
@@ -51152,7 +51158,7 @@
         <v>99</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>2340</v>
+        <v>2342</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>2310</v>
@@ -51161,13 +51167,13 @@
         <v>921</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>2353</v>
+        <v>2355</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>2349</v>
+        <v>2351</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>2354</v>
+        <v>2356</v>
       </c>
       <c r="I19" s="2">
         <v>24</v>
@@ -51184,22 +51190,22 @@
         <v>172</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>2355</v>
+        <v>2357</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>2356</v>
+        <v>2358</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>2357</v>
+        <v>2359</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="I20" s="2">
         <v>9</v>
@@ -51216,7 +51222,7 @@
         <v>1213</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>2358</v>
+        <v>2360</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>2310</v>
@@ -51225,13 +51231,13 @@
         <v>921</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>2348</v>
+        <v>2350</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>2359</v>
+        <v>2361</v>
       </c>
       <c r="I21" s="2">
         <v>6</v>
@@ -51248,22 +51254,22 @@
         <v>1268</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>2358</v>
+        <v>2360</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>2360</v>
+        <v>2362</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>2361</v>
+        <v>2363</v>
       </c>
       <c r="I22" s="2">
         <v>4</v>
@@ -51280,7 +51286,7 @@
         <v>1179</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>2358</v>
+        <v>2360</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>2310</v>
@@ -51289,13 +51295,13 @@
         <v>921</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>2348</v>
+        <v>2350</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>2362</v>
+        <v>2364</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>2363</v>
+        <v>2365</v>
       </c>
       <c r="I23" s="2">
         <v>16</v>
@@ -51330,7 +51336,7 @@
         <v>33</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2364</v>
+        <v>2366</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>41</v>
@@ -51351,36 +51357,36 @@
         <v>46</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>2365</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="2" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>2366</v>
+        <v>2368</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>2368</v>
+        <v>2370</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>2369</v>
+        <v>2371</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>2370</v>
+        <v>2372</v>
       </c>
       <c r="F2" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G2" s="15" t="s">
-        <v>2371</v>
+        <v>2373</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>2372</v>
+        <v>2374</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>2373</v>
+        <v>2375</v>
       </c>
       <c r="J2" s="2">
         <v>35</v>
@@ -51388,13 +51394,13 @@
     </row>
     <row r="3" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>2374</v>
+        <v>2376</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>2375</v>
+        <v>2377</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>63</v>
@@ -51420,13 +51426,13 @@
     </row>
     <row r="4" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>2376</v>
+        <v>2378</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>2377</v>
+        <v>2379</v>
       </c>
       <c r="D4" s="10" t="s">
         <v>63</v>
@@ -51452,19 +51458,19 @@
     </row>
     <row r="5" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>2378</v>
+        <v>2380</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>2379</v>
+        <v>2381</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>2380</v>
+        <v>2382</v>
       </c>
       <c r="F5" s="10" t="s">
         <v>63</v>
@@ -51484,16 +51490,16 @@
     </row>
     <row r="6" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>2381</v>
+        <v>2383</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>2382</v>
+        <v>2384</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>2383</v>
+        <v>2385</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>63</v>
@@ -51516,16 +51522,16 @@
     </row>
     <row r="7" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>2384</v>
+        <v>2386</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>2385</v>
+        <v>2387</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>2386</v>
+        <v>2388</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>63</v>
@@ -51534,10 +51540,10 @@
         <v>63</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>2387</v>
+        <v>2389</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>2388</v>
+        <v>2390</v>
       </c>
       <c r="I7" s="10" t="s">
         <v>63</v>
@@ -51548,19 +51554,19 @@
     </row>
     <row r="8" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>2389</v>
+        <v>2391</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>2390</v>
+        <v>2392</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>2391</v>
+        <v>2393</v>
       </c>
       <c r="F8" s="10" t="s">
         <v>63</v>
@@ -51580,19 +51586,19 @@
     </row>
     <row r="9" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>2392</v>
+        <v>2394</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>2393</v>
+        <v>2395</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>2394</v>
+        <v>2396</v>
       </c>
       <c r="F9" s="10" t="s">
         <v>63</v>
@@ -51612,16 +51618,16 @@
     </row>
     <row r="10" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>2395</v>
+        <v>2397</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>2397</v>
+        <v>2399</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>63</v>
@@ -51636,7 +51642,7 @@
         <v>63</v>
       </c>
       <c r="I10" s="15" t="s">
-        <v>2398</v>
+        <v>2400</v>
       </c>
       <c r="J10" s="2">
         <v>6</v>
@@ -51644,16 +51650,16 @@
     </row>
     <row r="11" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>2399</v>
+        <v>2401</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>2400</v>
+        <v>2402</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>2401</v>
+        <v>2403</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>63</v>
@@ -51662,7 +51668,7 @@
         <v>63</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>2402</v>
+        <v>2404</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>63</v>
@@ -51676,13 +51682,13 @@
     </row>
     <row r="12" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>2403</v>
+        <v>2405</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>2404</v>
+        <v>2406</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>63</v>
@@ -51694,7 +51700,7 @@
         <v>63</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>2405</v>
+        <v>2407</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>63</v>
@@ -51708,22 +51714,22 @@
     </row>
     <row r="13" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>2406</v>
+        <v>2408</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>2408</v>
+        <v>2410</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>2409</v>
+        <v>2411</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>2410</v>
+        <v>2412</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>2411</v>
+        <v>2413</v>
       </c>
       <c r="G13" s="10" t="s">
         <v>63</v>
@@ -51732,7 +51738,7 @@
         <v>63</v>
       </c>
       <c r="I13" s="15" t="s">
-        <v>2412</v>
+        <v>2414</v>
       </c>
       <c r="J13" s="2">
         <v>4</v>
@@ -51740,16 +51746,16 @@
     </row>
     <row r="14" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>2413</v>
+        <v>2415</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>2414</v>
+        <v>2416</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>2415</v>
+        <v>2417</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>63</v>
@@ -51764,7 +51770,7 @@
         <v>63</v>
       </c>
       <c r="I14" s="15" t="s">
-        <v>2416</v>
+        <v>2418</v>
       </c>
       <c r="J14" s="2">
         <v>9</v>
@@ -51772,31 +51778,31 @@
     </row>
     <row r="15" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>2417</v>
+        <v>2419</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>2418</v>
+        <v>2420</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>2419</v>
+        <v>2421</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>63</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>2420</v>
+        <v>2422</v>
       </c>
       <c r="G15" s="10" t="s">
         <v>63</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>2421</v>
+        <v>2423</v>
       </c>
       <c r="I15" s="15" t="s">
-        <v>2422</v>
+        <v>2424</v>
       </c>
       <c r="J15" s="2">
         <v>6</v>
@@ -51804,13 +51810,13 @@
     </row>
     <row r="16" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>2423</v>
+        <v>2425</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>2424</v>
+        <v>2426</v>
       </c>
       <c r="D16" s="10" t="s">
         <v>63</v>
@@ -51828,7 +51834,7 @@
         <v>63</v>
       </c>
       <c r="I16" s="15" t="s">
-        <v>2425</v>
+        <v>2427</v>
       </c>
       <c r="J16" s="2">
         <v>21</v>
@@ -51836,13 +51842,13 @@
     </row>
     <row r="17" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>2426</v>
+        <v>2428</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>2427</v>
+        <v>2429</v>
       </c>
       <c r="D17" s="10" t="s">
         <v>63</v>
@@ -51857,10 +51863,10 @@
         <v>63</v>
       </c>
       <c r="H17" s="15" t="s">
-        <v>2428</v>
+        <v>2430</v>
       </c>
       <c r="I17" s="15" t="s">
-        <v>2429</v>
+        <v>2431</v>
       </c>
       <c r="J17" s="2">
         <v>8</v>
@@ -51868,16 +51874,16 @@
     </row>
     <row r="18" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>2430</v>
+        <v>2432</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>2431</v>
+        <v>2433</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>2432</v>
+        <v>2434</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>63</v>
@@ -51886,13 +51892,13 @@
         <v>63</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>2433</v>
+        <v>2435</v>
       </c>
       <c r="H18" s="15" t="s">
-        <v>2434</v>
+        <v>2436</v>
       </c>
       <c r="I18" s="15" t="s">
-        <v>2435</v>
+        <v>2437</v>
       </c>
       <c r="J18" s="2">
         <v>5</v>
@@ -51900,16 +51906,16 @@
     </row>
     <row r="19" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>2436</v>
+        <v>2438</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>2437</v>
+        <v>2439</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>2438</v>
+        <v>2440</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>63</v>
@@ -51924,7 +51930,7 @@
         <v>63</v>
       </c>
       <c r="I19" s="15" t="s">
-        <v>2439</v>
+        <v>2441</v>
       </c>
       <c r="J19" s="2">
         <v>4</v>
@@ -51932,13 +51938,13 @@
     </row>
     <row r="20" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>2440</v>
+        <v>2442</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>2441</v>
+        <v>2443</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>63</v>
@@ -51956,7 +51962,7 @@
         <v>63</v>
       </c>
       <c r="I20" s="15" t="s">
-        <v>2442</v>
+        <v>2444</v>
       </c>
       <c r="J20" s="2">
         <v>2</v>
@@ -51964,16 +51970,16 @@
     </row>
     <row r="21" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>2443</v>
+        <v>2445</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>2444</v>
+        <v>2446</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>2445</v>
+        <v>2447</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>63</v>
@@ -51985,7 +51991,7 @@
         <v>63</v>
       </c>
       <c r="H21" s="16" t="s">
-        <v>2446</v>
+        <v>2448</v>
       </c>
       <c r="I21" s="10" t="s">
         <v>63</v>
@@ -51996,13 +52002,13 @@
     </row>
     <row r="22" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>2447</v>
+        <v>2449</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>2448</v>
+        <v>2450</v>
       </c>
       <c r="D22" s="10" t="s">
         <v>63</v>
@@ -52014,10 +52020,10 @@
         <v>63</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>2449</v>
+        <v>2451</v>
       </c>
       <c r="H22" s="15" t="s">
-        <v>2450</v>
+        <v>2452</v>
       </c>
       <c r="I22" s="10" t="s">
         <v>63</v>
@@ -52028,16 +52034,16 @@
     </row>
     <row r="23" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>2451</v>
+        <v>2453</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>2452</v>
+        <v>2454</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>2453</v>
+        <v>2455</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>63</v>
@@ -52060,13 +52066,13 @@
     </row>
     <row r="24" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>2454</v>
+        <v>2456</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>2455</v>
+        <v>2457</v>
       </c>
       <c r="D24" s="10" t="s">
         <v>63</v>
@@ -52084,7 +52090,7 @@
         <v>63</v>
       </c>
       <c r="I24" s="15" t="s">
-        <v>2456</v>
+        <v>2458</v>
       </c>
       <c r="J24" s="2">
         <v>0</v>
@@ -52092,31 +52098,31 @@
     </row>
     <row r="25" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>2457</v>
+        <v>2459</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>2458</v>
+        <v>2460</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>2459</v>
+        <v>2461</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>2432</v>
+        <v>2434</v>
       </c>
       <c r="E25" s="16" t="s">
-        <v>2460</v>
+        <v>2462</v>
       </c>
       <c r="F25" s="16" t="s">
-        <v>2461</v>
+        <v>2463</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>2433</v>
+        <v>2435</v>
       </c>
       <c r="H25" s="15" t="s">
-        <v>2462</v>
+        <v>2464</v>
       </c>
       <c r="I25" s="15" t="s">
-        <v>2463</v>
+        <v>2465</v>
       </c>
       <c r="J25" s="2">
         <v>25</v>
@@ -52124,16 +52130,16 @@
     </row>
     <row r="26" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>2464</v>
+        <v>2466</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>2458</v>
+        <v>2460</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>2465</v>
+        <v>2467</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>2466</v>
+        <v>2468</v>
       </c>
       <c r="E26" s="10" t="s">
         <v>63</v>
@@ -52156,19 +52162,19 @@
     </row>
     <row r="27" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>2467</v>
+        <v>2469</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>2458</v>
+        <v>2460</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>2468</v>
+        <v>2470</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>2469</v>
+        <v>2471</v>
       </c>
       <c r="E27" s="16" t="s">
-        <v>2470</v>
+        <v>2472</v>
       </c>
       <c r="F27" s="10" t="s">
         <v>63</v>
@@ -52177,7 +52183,7 @@
         <v>63</v>
       </c>
       <c r="H27" s="15" t="s">
-        <v>2471</v>
+        <v>2473</v>
       </c>
       <c r="I27" s="10" t="s">
         <v>63</v>
@@ -52188,19 +52194,19 @@
     </row>
     <row r="28" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>2472</v>
+        <v>2474</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>2458</v>
+        <v>2460</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>2473</v>
+        <v>2475</v>
       </c>
       <c r="D28" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>2474</v>
+        <v>2476</v>
       </c>
       <c r="F28" s="10" t="s">
         <v>63</v>
@@ -52220,16 +52226,16 @@
     </row>
     <row r="29" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>2475</v>
+        <v>2477</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>2458</v>
+        <v>2460</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>2476</v>
+        <v>2478</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>2477</v>
+        <v>2479</v>
       </c>
       <c r="E29" s="10" t="s">
         <v>63</v>
@@ -52252,16 +52258,16 @@
     </row>
     <row r="30" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>2478</v>
+        <v>2480</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>2458</v>
+        <v>2460</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>2479</v>
+        <v>2481</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>2480</v>
+        <v>2482</v>
       </c>
       <c r="E30" s="10" t="s">
         <v>63</v>
@@ -52276,7 +52282,7 @@
         <v>63</v>
       </c>
       <c r="I30" s="15" t="s">
-        <v>2481</v>
+        <v>2483</v>
       </c>
       <c r="J30" s="2">
         <v>12</v>
@@ -52284,31 +52290,31 @@
     </row>
     <row r="31" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>2482</v>
+        <v>2484</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>2484</v>
+        <v>2486</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>2485</v>
+        <v>2487</v>
       </c>
       <c r="E31" s="15" t="s">
-        <v>2486</v>
+        <v>2488</v>
       </c>
       <c r="F31" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G31" s="15" t="s">
-        <v>2487</v>
+        <v>2489</v>
       </c>
       <c r="H31" s="15" t="s">
-        <v>2488</v>
+        <v>2490</v>
       </c>
       <c r="I31" s="15" t="s">
-        <v>2489</v>
+        <v>2491</v>
       </c>
       <c r="J31" s="2">
         <v>5</v>
@@ -52316,19 +52322,19 @@
     </row>
     <row r="32" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>2490</v>
+        <v>2492</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>2491</v>
+        <v>2493</v>
       </c>
       <c r="D32" s="16" t="s">
-        <v>2492</v>
+        <v>2494</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>2493</v>
+        <v>2495</v>
       </c>
       <c r="F32" s="10" t="s">
         <v>63</v>
@@ -52337,10 +52343,10 @@
         <v>63</v>
       </c>
       <c r="H32" s="15" t="s">
-        <v>2494</v>
+        <v>2496</v>
       </c>
       <c r="I32" s="15" t="s">
-        <v>2495</v>
+        <v>2497</v>
       </c>
       <c r="J32" s="2">
         <v>4</v>
@@ -52348,25 +52354,25 @@
     </row>
     <row r="33" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>2496</v>
+        <v>2498</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>2497</v>
+        <v>2499</v>
       </c>
       <c r="D33" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E33" s="15" t="s">
-        <v>2498</v>
+        <v>2500</v>
       </c>
       <c r="F33" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G33" s="15" t="s">
-        <v>2499</v>
+        <v>2501</v>
       </c>
       <c r="H33" s="10" t="s">
         <v>63</v>
@@ -52380,19 +52386,19 @@
     </row>
     <row r="34" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>2500</v>
+        <v>2502</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>2501</v>
+        <v>2503</v>
       </c>
       <c r="D34" s="16" t="s">
-        <v>2492</v>
+        <v>2494</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>2502</v>
+        <v>2504</v>
       </c>
       <c r="F34" s="10" t="s">
         <v>63</v>
@@ -52404,7 +52410,7 @@
         <v>63</v>
       </c>
       <c r="I34" s="15" t="s">
-        <v>2503</v>
+        <v>2505</v>
       </c>
       <c r="J34" s="2">
         <v>0</v>
@@ -52412,16 +52418,16 @@
     </row>
     <row r="35" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>2504</v>
+        <v>2506</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>2505</v>
+        <v>2507</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>2506</v>
+        <v>2508</v>
       </c>
       <c r="E35" s="10" t="s">
         <v>63</v>
@@ -52444,19 +52450,19 @@
     </row>
     <row r="36" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>2507</v>
+        <v>2509</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>2508</v>
+        <v>2510</v>
       </c>
       <c r="D36" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E36" s="15" t="s">
-        <v>2509</v>
+        <v>2511</v>
       </c>
       <c r="F36" s="10" t="s">
         <v>63</v>
@@ -52476,19 +52482,19 @@
     </row>
     <row r="37" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>2510</v>
+        <v>2512</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>2511</v>
+        <v>2513</v>
       </c>
       <c r="D37" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E37" s="15" t="s">
-        <v>2512</v>
+        <v>2514</v>
       </c>
       <c r="F37" s="10" t="s">
         <v>63</v>
@@ -52508,13 +52514,13 @@
     </row>
     <row r="38" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>2513</v>
+        <v>2515</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>2514</v>
+        <v>2516</v>
       </c>
       <c r="D38" s="10" t="s">
         <v>63</v>
@@ -52532,7 +52538,7 @@
         <v>63</v>
       </c>
       <c r="I38" s="15" t="s">
-        <v>2515</v>
+        <v>2517</v>
       </c>
       <c r="J38" s="2">
         <v>0</v>
@@ -52540,13 +52546,13 @@
     </row>
     <row r="39" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>2516</v>
+        <v>2518</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>2517</v>
+        <v>2519</v>
       </c>
       <c r="D39" s="10" t="s">
         <v>63</v>
@@ -52564,7 +52570,7 @@
         <v>63</v>
       </c>
       <c r="I39" s="15" t="s">
-        <v>2518</v>
+        <v>2520</v>
       </c>
       <c r="J39" s="2">
         <v>12</v>
@@ -52572,13 +52578,13 @@
     </row>
     <row r="40" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>2519</v>
+        <v>2521</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>2520</v>
+        <v>2522</v>
       </c>
       <c r="D40" s="10" t="s">
         <v>63</v>
@@ -52596,7 +52602,7 @@
         <v>63</v>
       </c>
       <c r="I40" s="15" t="s">
-        <v>2521</v>
+        <v>2523</v>
       </c>
       <c r="J40" s="2">
         <v>0</v>
@@ -52604,31 +52610,31 @@
     </row>
     <row r="41" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>2522</v>
+        <v>2524</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>2523</v>
+        <v>2525</v>
       </c>
       <c r="D41" s="15" t="s">
-        <v>2524</v>
+        <v>2526</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>2525</v>
+        <v>2527</v>
       </c>
       <c r="F41" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G41" s="15" t="s">
-        <v>2526</v>
+        <v>2528</v>
       </c>
       <c r="H41" s="10" t="s">
         <v>63</v>
       </c>
       <c r="I41" s="15" t="s">
-        <v>2527</v>
+        <v>2529</v>
       </c>
       <c r="J41" s="2">
         <v>1</v>
@@ -52636,19 +52642,19 @@
     </row>
     <row r="42" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>2528</v>
+        <v>2530</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>2529</v>
+        <v>2531</v>
       </c>
       <c r="D42" s="15" t="s">
-        <v>2530</v>
+        <v>2532</v>
       </c>
       <c r="E42" s="15" t="s">
-        <v>2531</v>
+        <v>2533</v>
       </c>
       <c r="F42" s="10" t="s">
         <v>63</v>
@@ -52668,31 +52674,31 @@
     </row>
     <row r="43" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>2532</v>
+        <v>2534</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>2533</v>
+        <v>2535</v>
       </c>
       <c r="D43" s="15" t="s">
-        <v>2534</v>
+        <v>2536</v>
       </c>
       <c r="E43" s="15" t="s">
-        <v>2535</v>
+        <v>2537</v>
       </c>
       <c r="F43" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G43" s="15" t="s">
-        <v>2536</v>
+        <v>2538</v>
       </c>
       <c r="H43" s="15" t="s">
-        <v>2537</v>
+        <v>2539</v>
       </c>
       <c r="I43" s="15" t="s">
-        <v>2538</v>
+        <v>2540</v>
       </c>
       <c r="J43" s="2">
         <v>2</v>
@@ -52700,16 +52706,16 @@
     </row>
     <row r="44" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>2539</v>
+        <v>2541</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>2540</v>
+        <v>2542</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>2541</v>
+        <v>2543</v>
       </c>
       <c r="E44" s="10" t="s">
         <v>63</v>
@@ -52718,13 +52724,13 @@
         <v>63</v>
       </c>
       <c r="G44" s="15" t="s">
-        <v>2542</v>
+        <v>2544</v>
       </c>
       <c r="H44" s="10" t="s">
         <v>63</v>
       </c>
       <c r="I44" s="15" t="s">
-        <v>2543</v>
+        <v>2545</v>
       </c>
       <c r="J44" s="2">
         <v>4</v>
@@ -52732,31 +52738,31 @@
     </row>
     <row r="45" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>2544</v>
+        <v>2546</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>2545</v>
+        <v>2547</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>2546</v>
+        <v>2548</v>
       </c>
       <c r="D45" s="15" t="s">
-        <v>2547</v>
+        <v>2549</v>
       </c>
       <c r="E45" s="15" t="s">
-        <v>2548</v>
+        <v>2550</v>
       </c>
       <c r="F45" s="16" t="s">
-        <v>2549</v>
+        <v>2551</v>
       </c>
       <c r="G45" s="15" t="s">
-        <v>2550</v>
+        <v>2552</v>
       </c>
       <c r="H45" s="15" t="s">
-        <v>2551</v>
+        <v>2553</v>
       </c>
       <c r="I45" s="9" t="s">
-        <v>2552</v>
+        <v>2554</v>
       </c>
       <c r="J45" s="2">
         <v>3</v>
@@ -52764,31 +52770,31 @@
     </row>
     <row r="46" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>2553</v>
+        <v>2555</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>2545</v>
+        <v>2547</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>2554</v>
+        <v>2556</v>
       </c>
       <c r="D46" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E46" s="15" t="s">
-        <v>2555</v>
+        <v>2557</v>
       </c>
       <c r="F46" s="15" t="s">
-        <v>2556</v>
+        <v>2558</v>
       </c>
       <c r="G46" s="10" t="s">
         <v>63</v>
       </c>
       <c r="H46" s="15" t="s">
-        <v>2557</v>
+        <v>2559</v>
       </c>
       <c r="I46" s="15" t="s">
-        <v>2558</v>
+        <v>2560</v>
       </c>
       <c r="J46" s="2">
         <v>3</v>
@@ -52796,25 +52802,25 @@
     </row>
     <row r="47" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>2559</v>
+        <v>2561</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>2545</v>
+        <v>2547</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>2560</v>
+        <v>2562</v>
       </c>
       <c r="D47" s="15" t="s">
-        <v>2561</v>
+        <v>2563</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>2562</v>
+        <v>2564</v>
       </c>
       <c r="F47" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G47" s="15" t="s">
-        <v>2563</v>
+        <v>2565</v>
       </c>
       <c r="H47" s="10" t="s">
         <v>63</v>
@@ -52828,13 +52834,13 @@
     </row>
     <row r="48" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>2564</v>
+        <v>2566</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>2545</v>
+        <v>2547</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>2565</v>
+        <v>2567</v>
       </c>
       <c r="D48" s="10" t="s">
         <v>63</v>
@@ -52846,10 +52852,10 @@
         <v>63</v>
       </c>
       <c r="G48" s="15" t="s">
-        <v>2566</v>
+        <v>2568</v>
       </c>
       <c r="H48" s="15" t="s">
-        <v>2567</v>
+        <v>2569</v>
       </c>
       <c r="I48" s="10" t="s">
         <v>63</v>
@@ -52860,13 +52866,13 @@
     </row>
     <row r="49" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>2568</v>
+        <v>2570</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>2545</v>
+        <v>2547</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>2569</v>
+        <v>2571</v>
       </c>
       <c r="D49" s="10" t="s">
         <v>63</v>
@@ -52881,10 +52887,10 @@
         <v>63</v>
       </c>
       <c r="H49" s="15" t="s">
-        <v>2570</v>
+        <v>2572</v>
       </c>
       <c r="I49" s="15" t="s">
-        <v>2571</v>
+        <v>2573</v>
       </c>
       <c r="J49" s="2">
         <v>15</v>
@@ -52892,13 +52898,13 @@
     </row>
     <row r="50" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>2572</v>
+        <v>2574</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>2573</v>
+        <v>2575</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>2574</v>
+        <v>2576</v>
       </c>
       <c r="D50" s="10" t="s">
         <v>63</v>
@@ -52913,7 +52919,7 @@
         <v>63</v>
       </c>
       <c r="H50" s="15" t="s">
-        <v>2575</v>
+        <v>2577</v>
       </c>
       <c r="I50" s="10" t="s">
         <v>63</v>
@@ -52924,13 +52930,13 @@
     </row>
     <row r="51" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>2576</v>
+        <v>2578</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>2545</v>
+        <v>2547</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>2577</v>
+        <v>2579</v>
       </c>
       <c r="D51" s="10" t="s">
         <v>63</v>
@@ -52945,7 +52951,7 @@
         <v>63</v>
       </c>
       <c r="H51" s="16" t="s">
-        <v>2578</v>
+        <v>2580</v>
       </c>
       <c r="I51" s="10" t="s">
         <v>63</v>
@@ -52956,13 +52962,13 @@
     </row>
     <row r="52" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>2579</v>
+        <v>2581</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>2573</v>
+        <v>2575</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>2580</v>
+        <v>2582</v>
       </c>
       <c r="D52" s="10" t="s">
         <v>63</v>
@@ -52977,7 +52983,7 @@
         <v>63</v>
       </c>
       <c r="H52" s="15" t="s">
-        <v>2581</v>
+        <v>2583</v>
       </c>
       <c r="I52" s="10" t="s">
         <v>63</v>
@@ -52988,13 +52994,13 @@
     </row>
     <row r="53" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>2582</v>
+        <v>2584</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>2545</v>
+        <v>2547</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>2583</v>
+        <v>2585</v>
       </c>
       <c r="D53" s="10" t="s">
         <v>63</v>
@@ -53009,7 +53015,7 @@
         <v>63</v>
       </c>
       <c r="H53" s="15" t="s">
-        <v>2584</v>
+        <v>2586</v>
       </c>
       <c r="I53" s="10" t="s">
         <v>63</v>
@@ -53020,19 +53026,19 @@
     </row>
     <row r="54" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>2585</v>
+        <v>2587</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>2586</v>
+        <v>2588</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>2587</v>
+        <v>2589</v>
       </c>
       <c r="D54" s="15" t="s">
-        <v>2588</v>
+        <v>2590</v>
       </c>
       <c r="E54" s="15" t="s">
-        <v>2589</v>
+        <v>2591</v>
       </c>
       <c r="F54" s="10" t="s">
         <v>63</v>
@@ -53052,19 +53058,19 @@
     </row>
     <row r="55" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>2590</v>
+        <v>2592</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>2586</v>
+        <v>2588</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>2591</v>
+        <v>2593</v>
       </c>
       <c r="D55" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E55" s="15" t="s">
-        <v>2592</v>
+        <v>2594</v>
       </c>
       <c r="F55" s="10" t="s">
         <v>63</v>
@@ -53084,19 +53090,19 @@
     </row>
     <row r="56" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>2593</v>
+        <v>2595</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>2586</v>
+        <v>2588</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>2594</v>
+        <v>2596</v>
       </c>
       <c r="D56" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E56" s="15" t="s">
-        <v>2595</v>
+        <v>2597</v>
       </c>
       <c r="F56" s="10" t="s">
         <v>63</v>
@@ -53116,28 +53122,28 @@
     </row>
     <row r="57" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>2596</v>
+        <v>2598</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>2597</v>
+        <v>2599</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>2598</v>
+        <v>2600</v>
       </c>
       <c r="D57" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E57" s="15" t="s">
-        <v>2599</v>
+        <v>2601</v>
       </c>
       <c r="F57" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G57" s="15" t="s">
-        <v>2600</v>
+        <v>2602</v>
       </c>
       <c r="H57" s="15" t="s">
-        <v>2601</v>
+        <v>2603</v>
       </c>
       <c r="I57" s="10" t="s">
         <v>63</v>
@@ -53148,13 +53154,13 @@
     </row>
     <row r="58" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>2602</v>
+        <v>2604</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>2597</v>
+        <v>2599</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>2603</v>
+        <v>2605</v>
       </c>
       <c r="D58" s="10" t="s">
         <v>63</v>
@@ -53169,7 +53175,7 @@
         <v>63</v>
       </c>
       <c r="H58" s="15" t="s">
-        <v>2604</v>
+        <v>2606</v>
       </c>
       <c r="I58" s="10" t="s">
         <v>63</v>
@@ -53180,19 +53186,19 @@
     </row>
     <row r="59" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>2605</v>
+        <v>2607</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>2597</v>
+        <v>2599</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>2606</v>
+        <v>2608</v>
       </c>
       <c r="D59" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>2607</v>
+        <v>2609</v>
       </c>
       <c r="F59" s="10" t="s">
         <v>63</v>
@@ -53201,7 +53207,7 @@
         <v>63</v>
       </c>
       <c r="H59" s="15" t="s">
-        <v>2608</v>
+        <v>2610</v>
       </c>
       <c r="I59" s="10" t="s">
         <v>63</v>
@@ -53212,19 +53218,19 @@
     </row>
     <row r="60" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>2609</v>
+        <v>2611</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>2597</v>
+        <v>2599</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>2610</v>
+        <v>2612</v>
       </c>
       <c r="D60" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E60" s="15" t="s">
-        <v>2611</v>
+        <v>2613</v>
       </c>
       <c r="F60" s="10" t="s">
         <v>63</v>
@@ -53233,7 +53239,7 @@
         <v>63</v>
       </c>
       <c r="H60" s="15" t="s">
-        <v>2612</v>
+        <v>2614</v>
       </c>
       <c r="I60" s="10" t="s">
         <v>63</v>
@@ -53244,19 +53250,19 @@
     </row>
     <row r="61" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>2613</v>
+        <v>2615</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>2597</v>
+        <v>2599</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>2614</v>
+        <v>2616</v>
       </c>
       <c r="D61" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E61" s="15" t="s">
-        <v>2615</v>
+        <v>2617</v>
       </c>
       <c r="F61" s="10" t="s">
         <v>63</v>
@@ -53276,25 +53282,25 @@
     </row>
     <row r="62" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>2616</v>
+        <v>2618</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>2617</v>
+        <v>2619</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>2618</v>
+        <v>2620</v>
       </c>
       <c r="D62" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E62" s="9" t="s">
-        <v>2619</v>
+        <v>2621</v>
       </c>
       <c r="F62" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G62" s="9" t="s">
-        <v>2620</v>
+        <v>2622</v>
       </c>
       <c r="H62" s="10" t="s">
         <v>63</v>
@@ -53308,31 +53314,31 @@
     </row>
     <row r="63" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>2621</v>
+        <v>2623</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>2622</v>
+        <v>2624</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>2623</v>
+        <v>2625</v>
       </c>
       <c r="D63" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E63" s="15" t="s">
-        <v>2624</v>
+        <v>2626</v>
       </c>
       <c r="F63" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G63" s="15" t="s">
-        <v>2625</v>
+        <v>2627</v>
       </c>
       <c r="H63" s="10" t="s">
         <v>63</v>
       </c>
       <c r="I63" s="15" t="s">
-        <v>2626</v>
+        <v>2628</v>
       </c>
       <c r="J63" s="2">
         <v>4</v>
@@ -53340,13 +53346,13 @@
     </row>
     <row r="64" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>2627</v>
+        <v>2629</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>2622</v>
+        <v>2624</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>2628</v>
+        <v>2630</v>
       </c>
       <c r="D64" s="10" t="s">
         <v>63</v>
@@ -53358,7 +53364,7 @@
         <v>63</v>
       </c>
       <c r="G64" s="15" t="s">
-        <v>2629</v>
+        <v>2631</v>
       </c>
       <c r="H64" s="10" t="s">
         <v>63</v>
@@ -53372,25 +53378,25 @@
     </row>
     <row r="65" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>2630</v>
+        <v>2632</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>2622</v>
+        <v>2624</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>2631</v>
+        <v>2633</v>
       </c>
       <c r="D65" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E65" s="15" t="s">
-        <v>2632</v>
+        <v>2634</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G65" s="15" t="s">
-        <v>2633</v>
+        <v>2635</v>
       </c>
       <c r="H65" s="10" t="s">
         <v>63</v>
@@ -53404,13 +53410,13 @@
     </row>
     <row r="66" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>2634</v>
+        <v>2636</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>2635</v>
+        <v>2637</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>2636</v>
+        <v>2638</v>
       </c>
       <c r="D66" s="10" t="s">
         <v>63</v>
@@ -53422,7 +53428,7 @@
         <v>63</v>
       </c>
       <c r="G66" s="15" t="s">
-        <v>2637</v>
+        <v>2639</v>
       </c>
       <c r="H66" s="10" t="s">
         <v>63</v>
@@ -53436,19 +53442,19 @@
     </row>
     <row r="67" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>2638</v>
+        <v>2640</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>2635</v>
+        <v>2637</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>2639</v>
+        <v>2641</v>
       </c>
       <c r="D67" s="16" t="s">
-        <v>2640</v>
+        <v>2642</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>2641</v>
+        <v>2643</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>63</v>
@@ -53468,13 +53474,13 @@
     </row>
     <row r="68" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>2642</v>
+        <v>2644</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>2635</v>
+        <v>2637</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>2643</v>
+        <v>2645</v>
       </c>
       <c r="D68" s="10" t="s">
         <v>63</v>
@@ -53483,7 +53489,7 @@
         <v>63</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>2644</v>
+        <v>2646</v>
       </c>
       <c r="G68" s="10" t="s">
         <v>63</v>
@@ -53500,13 +53506,13 @@
     </row>
     <row r="69" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>2645</v>
+        <v>2647</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>2646</v>
+        <v>2648</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>2647</v>
+        <v>2649</v>
       </c>
       <c r="D69" s="10" t="s">
         <v>63</v>
@@ -53521,7 +53527,7 @@
         <v>63</v>
       </c>
       <c r="H69" s="9" t="s">
-        <v>2648</v>
+        <v>2650</v>
       </c>
       <c r="I69" s="10" t="s">
         <v>63</v>
@@ -53532,13 +53538,13 @@
     </row>
     <row r="70" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>2649</v>
+        <v>2651</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>2646</v>
+        <v>2648</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>2650</v>
+        <v>2652</v>
       </c>
       <c r="D70" s="10" t="s">
         <v>63</v>
@@ -53553,7 +53559,7 @@
         <v>63</v>
       </c>
       <c r="H70" s="15" t="s">
-        <v>2651</v>
+        <v>2653</v>
       </c>
       <c r="I70" s="10" t="s">
         <v>63</v>
@@ -53564,13 +53570,13 @@
     </row>
     <row r="71" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>2652</v>
+        <v>2654</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>2654</v>
+        <v>2656</v>
       </c>
       <c r="D71" s="10" t="s">
         <v>63</v>
@@ -53585,7 +53591,7 @@
         <v>63</v>
       </c>
       <c r="H71" s="15" t="s">
-        <v>2655</v>
+        <v>2657</v>
       </c>
       <c r="I71" s="10" t="s">
         <v>63</v>
@@ -53596,13 +53602,13 @@
     </row>
     <row r="72" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>2656</v>
+        <v>2658</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>2657</v>
+        <v>2659</v>
       </c>
       <c r="D72" s="10" t="s">
         <v>63</v>
@@ -53617,7 +53623,7 @@
         <v>63</v>
       </c>
       <c r="H72" s="15" t="s">
-        <v>2658</v>
+        <v>2660</v>
       </c>
       <c r="I72" s="10" t="s">
         <v>63</v>
@@ -53628,13 +53634,13 @@
     </row>
     <row r="73" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>2659</v>
+        <v>2661</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>2660</v>
+        <v>2662</v>
       </c>
       <c r="D73" s="10" t="s">
         <v>63</v>
@@ -53649,7 +53655,7 @@
         <v>63</v>
       </c>
       <c r="H73" s="15" t="s">
-        <v>2661</v>
+        <v>2663</v>
       </c>
       <c r="I73" s="10" t="s">
         <v>63</v>
@@ -53660,19 +53666,19 @@
     </row>
     <row r="74" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>2662</v>
+        <v>2664</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>2663</v>
+        <v>2665</v>
       </c>
       <c r="D74" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E74" s="9" t="s">
-        <v>2664</v>
+        <v>2666</v>
       </c>
       <c r="F74" s="10" t="s">
         <v>63</v>
@@ -53681,7 +53687,7 @@
         <v>63</v>
       </c>
       <c r="H74" s="15" t="s">
-        <v>2665</v>
+        <v>2667</v>
       </c>
       <c r="I74" s="10" t="s">
         <v>63</v>
@@ -53692,13 +53698,13 @@
     </row>
     <row r="75" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>2666</v>
+        <v>2668</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>2646</v>
+        <v>2648</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>2667</v>
+        <v>2669</v>
       </c>
       <c r="D75" s="10" t="s">
         <v>63</v>
@@ -53713,7 +53719,7 @@
         <v>63</v>
       </c>
       <c r="H75" s="15" t="s">
-        <v>2668</v>
+        <v>2670</v>
       </c>
       <c r="I75" s="10" t="s">
         <v>63</v>
@@ -53724,13 +53730,13 @@
     </row>
     <row r="76" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>2669</v>
+        <v>2671</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>2670</v>
+        <v>2672</v>
       </c>
       <c r="D76" s="10" t="s">
         <v>63</v>
@@ -53745,7 +53751,7 @@
         <v>63</v>
       </c>
       <c r="H76" s="9" t="s">
-        <v>2671</v>
+        <v>2673</v>
       </c>
       <c r="I76" s="10" t="s">
         <v>63</v>
@@ -53756,13 +53762,13 @@
     </row>
     <row r="77" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>2672</v>
+        <v>2674</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>2673</v>
+        <v>2675</v>
       </c>
       <c r="D77" s="10" t="s">
         <v>63</v>
@@ -53777,7 +53783,7 @@
         <v>63</v>
       </c>
       <c r="H77" s="15" t="s">
-        <v>2674</v>
+        <v>2676</v>
       </c>
       <c r="I77" s="10" t="s">
         <v>63</v>
@@ -53788,13 +53794,13 @@
     </row>
     <row r="78" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>2675</v>
+        <v>2677</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>2676</v>
+        <v>2678</v>
       </c>
       <c r="D78" s="10" t="s">
         <v>63</v>
@@ -53809,7 +53815,7 @@
         <v>63</v>
       </c>
       <c r="H78" s="15" t="s">
-        <v>2677</v>
+        <v>2679</v>
       </c>
       <c r="I78" s="10" t="s">
         <v>63</v>
@@ -53820,19 +53826,19 @@
     </row>
     <row r="79" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>2678</v>
+        <v>2680</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>2679</v>
+        <v>2681</v>
       </c>
       <c r="D79" s="16" t="s">
-        <v>2680</v>
+        <v>2682</v>
       </c>
       <c r="E79" s="15" t="s">
-        <v>2681</v>
+        <v>2683</v>
       </c>
       <c r="F79" s="10" t="s">
         <v>63</v>
@@ -53841,7 +53847,7 @@
         <v>63</v>
       </c>
       <c r="H79" s="16" t="s">
-        <v>2680</v>
+        <v>2682</v>
       </c>
       <c r="I79" s="10" t="s">
         <v>63</v>
@@ -53852,13 +53858,13 @@
     </row>
     <row r="80" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>2682</v>
+        <v>2684</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>2683</v>
+        <v>2685</v>
       </c>
       <c r="D80" s="10" t="s">
         <v>63</v>
@@ -53873,7 +53879,7 @@
         <v>63</v>
       </c>
       <c r="H80" s="15" t="s">
-        <v>2684</v>
+        <v>2686</v>
       </c>
       <c r="I80" s="10" t="s">
         <v>63</v>
@@ -53884,13 +53890,13 @@
     </row>
     <row r="81" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>2685</v>
+        <v>2687</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>2686</v>
+        <v>2688</v>
       </c>
       <c r="D81" s="10" t="s">
         <v>63</v>
@@ -53905,7 +53911,7 @@
         <v>63</v>
       </c>
       <c r="H81" s="15" t="s">
-        <v>2687</v>
+        <v>2689</v>
       </c>
       <c r="I81" s="10" t="s">
         <v>63</v>
@@ -53916,13 +53922,13 @@
     </row>
     <row r="82" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>2688</v>
+        <v>2690</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>2689</v>
+        <v>2691</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>2690</v>
+        <v>2692</v>
       </c>
       <c r="D82" s="10" t="s">
         <v>63</v>
@@ -53937,7 +53943,7 @@
         <v>63</v>
       </c>
       <c r="H82" s="15" t="s">
-        <v>2691</v>
+        <v>2693</v>
       </c>
       <c r="I82" s="10" t="s">
         <v>63</v>
@@ -53948,19 +53954,19 @@
     </row>
     <row r="83" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>2692</v>
+        <v>2694</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>2693</v>
+        <v>2695</v>
       </c>
       <c r="D83" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E83" s="15" t="s">
-        <v>2694</v>
+        <v>2696</v>
       </c>
       <c r="F83" s="10" t="s">
         <v>63</v>
@@ -53969,7 +53975,7 @@
         <v>63</v>
       </c>
       <c r="H83" s="15" t="s">
-        <v>2695</v>
+        <v>2697</v>
       </c>
       <c r="I83" s="10" t="s">
         <v>63</v>
@@ -53980,13 +53986,13 @@
     </row>
     <row r="84" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>2696</v>
+        <v>2698</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>2635</v>
+        <v>2637</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>2697</v>
+        <v>2699</v>
       </c>
       <c r="D84" s="10" t="s">
         <v>63</v>
@@ -53995,7 +54001,7 @@
         <v>63</v>
       </c>
       <c r="F84" s="15" t="s">
-        <v>2698</v>
+        <v>2700</v>
       </c>
       <c r="G84" s="10" t="s">
         <v>63</v>
@@ -54012,13 +54018,13 @@
     </row>
     <row r="85" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>2699</v>
+        <v>2701</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>2700</v>
+        <v>2702</v>
       </c>
       <c r="D85" s="10" t="s">
         <v>63</v>
@@ -54036,7 +54042,7 @@
         <v>63</v>
       </c>
       <c r="I85" s="15" t="s">
-        <v>2701</v>
+        <v>2703</v>
       </c>
       <c r="J85" s="2">
         <v>0</v>
@@ -54044,31 +54050,31 @@
     </row>
     <row r="86" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>2702</v>
+        <v>2704</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>2703</v>
+        <v>2705</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>2704</v>
+        <v>2706</v>
       </c>
       <c r="D86" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E86" s="15" t="s">
-        <v>2705</v>
+        <v>2707</v>
       </c>
       <c r="F86" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G86" s="15" t="s">
-        <v>2706</v>
+        <v>2708</v>
       </c>
       <c r="H86" s="10" t="s">
         <v>63</v>
       </c>
       <c r="I86" s="15" t="s">
-        <v>2707</v>
+        <v>2709</v>
       </c>
       <c r="J86" s="2">
         <v>3</v>
@@ -54076,19 +54082,19 @@
     </row>
     <row r="87" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>2708</v>
+        <v>2710</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>2709</v>
+        <v>2711</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>2710</v>
+        <v>2712</v>
       </c>
       <c r="D87" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E87" s="15" t="s">
-        <v>2711</v>
+        <v>2713</v>
       </c>
       <c r="F87" s="10" t="s">
         <v>63</v>
@@ -54108,16 +54114,16 @@
     </row>
     <row r="88" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>2712</v>
+        <v>2714</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>2703</v>
+        <v>2705</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>2713</v>
+        <v>2715</v>
       </c>
       <c r="D88" s="15" t="s">
-        <v>2714</v>
+        <v>2716</v>
       </c>
       <c r="E88" s="10" t="s">
         <v>63</v>
@@ -54126,7 +54132,7 @@
         <v>63</v>
       </c>
       <c r="G88" s="15" t="s">
-        <v>2715</v>
+        <v>2717</v>
       </c>
       <c r="H88" s="10" t="s">
         <v>63</v>
@@ -54140,25 +54146,25 @@
     </row>
     <row r="89" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>2716</v>
+        <v>2718</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>2703</v>
+        <v>2705</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>2717</v>
+        <v>2719</v>
       </c>
       <c r="D89" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E89" s="15" t="s">
-        <v>2718</v>
+        <v>2720</v>
       </c>
       <c r="F89" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G89" s="9" t="s">
-        <v>2719</v>
+        <v>2721</v>
       </c>
       <c r="H89" s="10" t="s">
         <v>63</v>
@@ -54172,13 +54178,13 @@
     </row>
     <row r="90" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>2720</v>
+        <v>2722</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>2703</v>
+        <v>2705</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>2721</v>
+        <v>2723</v>
       </c>
       <c r="D90" s="10" t="s">
         <v>63</v>
@@ -54190,13 +54196,13 @@
         <v>63</v>
       </c>
       <c r="G90" s="15" t="s">
-        <v>2722</v>
+        <v>2724</v>
       </c>
       <c r="H90" s="15" t="s">
-        <v>2723</v>
+        <v>2725</v>
       </c>
       <c r="I90" s="15" t="s">
-        <v>2724</v>
+        <v>2726</v>
       </c>
       <c r="J90" s="2">
         <v>14</v>
@@ -54204,13 +54210,13 @@
     </row>
     <row r="91" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>2725</v>
+        <v>2727</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>2726</v>
+        <v>2728</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>2727</v>
+        <v>2729</v>
       </c>
       <c r="D91" s="10" t="s">
         <v>63</v>
@@ -54225,7 +54231,7 @@
         <v>63</v>
       </c>
       <c r="H91" s="15" t="s">
-        <v>2728</v>
+        <v>2730</v>
       </c>
       <c r="I91" s="10" t="s">
         <v>63</v>
@@ -54257,16 +54263,16 @@
         <v>32</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>2729</v>
+        <v>2731</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2730</v>
+        <v>2732</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>35</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>2731</v>
+        <v>2733</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -54274,16 +54280,16 @@
         <v>143</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>2732</v>
+        <v>2734</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>2733</v>
+        <v>2735</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>2734</v>
+        <v>2736</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>2735</v>
+        <v>2737</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -54291,16 +54297,16 @@
         <v>1340</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>2738</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>2739</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>2736</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>2737</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>2734</v>
-      </c>
       <c r="E3" s="2" t="s">
-        <v>2738</v>
+        <v>2740</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -54308,16 +54314,16 @@
         <v>110</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>2739</v>
+        <v>2741</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>2740</v>
+        <v>2742</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>2741</v>
+        <v>2743</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>2742</v>
+        <v>2744</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -54325,16 +54331,16 @@
         <v>920</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>2745</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>2746</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>2743</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>2744</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>2741</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>2735</v>
+        <v>2737</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -54342,16 +54348,16 @@
         <v>363</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>2745</v>
+        <v>2747</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>2746</v>
+        <v>2748</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>2734</v>
+        <v>2736</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>2735</v>
+        <v>2737</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -54359,16 +54365,16 @@
         <v>454</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>2747</v>
+        <v>2749</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>2748</v>
+        <v>2750</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>2734</v>
+        <v>2736</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>2735</v>
+        <v>2737</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -54376,16 +54382,16 @@
         <v>104</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>2749</v>
+        <v>2751</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>2750</v>
+        <v>2752</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>2734</v>
+        <v>2736</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>2751</v>
+        <v>2753</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -54393,33 +54399,33 @@
         <v>377</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>2752</v>
+        <v>2754</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>2753</v>
+        <v>2755</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>2734</v>
+        <v>2736</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>2735</v>
+        <v>2737</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>2754</v>
+        <v>2756</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>2755</v>
+        <v>2757</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>2756</v>
+        <v>2758</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>2734</v>
+        <v>2736</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>2735</v>
+        <v>2737</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -54427,59 +54433,59 @@
         <v>809</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>2757</v>
+        <v>2759</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>2758</v>
+        <v>2760</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>2759</v>
+        <v>2761</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>2760</v>
+        <v>2762</v>
       </c>
     </row>
     <row r="13" spans="2:2" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B13" s="17" t="s">
-        <v>2761</v>
+        <v>2763</v>
       </c>
     </row>
     <row r="14" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
-        <v>2762</v>
+        <v>2764</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>2763</v>
+        <v>2765</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>2764</v>
+        <v>2766</v>
       </c>
     </row>
     <row r="15" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
-        <v>2765</v>
+        <v>2767</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>2766</v>
+        <v>2768</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>2767</v>
+        <v>2769</v>
       </c>
     </row>
     <row r="16" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
-        <v>2768</v>
+        <v>2770</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>2769</v>
+        <v>2771</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>2770</v>
+        <v>2772</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>2771</v>
+        <v>2773</v>
       </c>
     </row>
   </sheetData>
@@ -54505,10 +54511,10 @@
         <v>33</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>2772</v>
+        <v>2774</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2773</v>
+        <v>2775</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>56</v>
@@ -54520,7 +54526,7 @@
         <v>64</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>2774</v>
+        <v>2776</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>102</v>
@@ -54540,7 +54546,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="B2" t="s">
         <v>51</v>
@@ -54578,7 +54584,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2646</v>
+        <v>2648</v>
       </c>
       <c r="B3" t="s">
         <v>397</v>
@@ -54616,7 +54622,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="B4" t="s">
         <v>541</v>
@@ -54654,7 +54660,7 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="B5" t="s">
         <v>702</v>
@@ -54692,7 +54698,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>2458</v>
+        <v>2460</v>
       </c>
       <c r="B6" t="s">
         <v>848</v>
@@ -54730,7 +54736,7 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="B7" t="s">
         <v>996</v>
@@ -54768,7 +54774,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>2573</v>
+        <v>2575</v>
       </c>
       <c r="B8" t="s">
         <v>1147</v>
@@ -54806,7 +54812,7 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>2545</v>
+        <v>2547</v>
       </c>
       <c r="B9" t="s">
         <v>1237</v>
@@ -54844,7 +54850,7 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>2586</v>
+        <v>2588</v>
       </c>
       <c r="B10" t="s">
         <v>1354</v>
@@ -54882,7 +54888,7 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>2597</v>
+        <v>2599</v>
       </c>
       <c r="B11" t="s">
         <v>1420</v>
@@ -54920,7 +54926,7 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>2617</v>
+        <v>2619</v>
       </c>
       <c r="B12" t="s">
         <v>1504</v>
@@ -54958,7 +54964,7 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>2635</v>
+        <v>2637</v>
       </c>
       <c r="B13" t="s">
         <v>1552</v>
@@ -54996,7 +55002,7 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>2689</v>
+        <v>2691</v>
       </c>
       <c r="B14" t="s">
         <v>1671</v>
@@ -55034,7 +55040,7 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>2622</v>
+        <v>2624</v>
       </c>
       <c r="B15" t="s">
         <v>1759</v>
@@ -55072,7 +55078,7 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>2703</v>
+        <v>2705</v>
       </c>
       <c r="B16" t="s">
         <v>1793</v>
@@ -55110,7 +55116,7 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>2775</v>
+        <v>2777</v>
       </c>
       <c r="B17" t="s">
         <v>1911</v>
@@ -55148,7 +55154,7 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>2726</v>
+        <v>2728</v>
       </c>
       <c r="B18" t="s">
         <v>1973</v>
@@ -55186,7 +55192,7 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>2776</v>
+        <v>2778</v>
       </c>
       <c r="B19" t="s">
         <v>2001</v>
@@ -55224,7 +55230,7 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>2709</v>
+        <v>2711</v>
       </c>
       <c r="B20" t="s">
         <v>2017</v>
@@ -55262,7 +55268,7 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>2777</v>
+        <v>2779</v>
       </c>
       <c r="B21" t="s">
         <v>2048</v>
@@ -55300,7 +55306,7 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>2778</v>
+        <v>2780</v>
       </c>
       <c r="B22" t="s">
         <v>2088</v>
@@ -55338,7 +55344,7 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>2779</v>
+        <v>2781</v>
       </c>
       <c r="B23" t="s">
         <v>2117</v>
@@ -55376,7 +55382,7 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>2780</v>
+        <v>2782</v>
       </c>
       <c r="B24" t="s">
         <v>2145</v>
@@ -55414,7 +55420,7 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>2781</v>
+        <v>2783</v>
       </c>
       <c r="B25" t="s">
         <v>2184</v>
@@ -55452,7 +55458,7 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>2782</v>
+        <v>2784</v>
       </c>
       <c r="B26" t="s">
         <v>2207</v>
@@ -55490,7 +55496,7 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>2783</v>
+        <v>2785</v>
       </c>
       <c r="B27" t="s">
         <v>2221</v>
@@ -55528,7 +55534,7 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>2784</v>
+        <v>2786</v>
       </c>
       <c r="B28" t="s">
         <v>2238</v>
@@ -55566,7 +55572,7 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>2785</v>
+        <v>2787</v>
       </c>
       <c r="B29" t="s">
         <v>2262</v>
@@ -55604,7 +55610,7 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>2786</v>
+        <v>2788</v>
       </c>
       <c r="B30" t="s">
         <v>2277</v>
@@ -55642,7 +55648,7 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>2787</v>
+        <v>2789</v>
       </c>
       <c r="B31" t="s">
         <v>2294</v>
@@ -55680,7 +55686,7 @@
     </row>
     <row r="33" spans="2:12" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B33" s="17" t="s">
-        <v>2773</v>
+        <v>2775</v>
       </c>
       <c r="C33" s="17">
         <v>559</v>

</xml_diff>

<commit_message>
docs: entrevistas de estudiantes E1–E4, estado de las necesidades y regla de no comentar en Asana
</commit_message>
<xml_diff>
--- a/docs/requisitos/FOOD4ALL_requisitos_benchmark.xlsx
+++ b/docs/requisitos/FOOD4ALL_requisitos_benchmark.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14618" uniqueCount="2788">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14618" uniqueCount="2790">
   <si>
     <t>FOOD4ALL · Catálogo de requisitos con benchmark</t>
   </si>
@@ -7031,7 +7031,10 @@
     <t>Usuario</t>
   </si>
   <si>
-    <t>F-01, F-02</t>
+    <t>Indicio</t>
+  </si>
+  <si>
+    <t>F-01, F-02, F-07 (E3, E4)</t>
   </si>
   <si>
     <t>N-01</t>
@@ -7040,10 +7043,10 @@
     <t>N-03, N-04, N-05</t>
   </si>
   <si>
-    <t>F-01</t>
-  </si>
-  <si>
-    <t>F-04, F-10</t>
+    <t>F-01, F-07 (E4; E1 comparativo)</t>
+  </si>
+  <si>
+    <t>F-04, F-10, F-07 (E4; E3 en contra del producto, no de la necesidad)</t>
   </si>
   <si>
     <t>N-02</t>
@@ -7058,7 +7061,7 @@
     <t>N-10</t>
   </si>
   <si>
-    <t>F-01, F-03</t>
+    <t>F-01, F-03, F-07 (E3, E4)</t>
   </si>
   <si>
     <t>N-08</t>
@@ -7067,7 +7070,10 @@
     <t>N-06, N-07</t>
   </si>
   <si>
-    <t>F-02</t>
+    <t>No confirmada</t>
+  </si>
+  <si>
+    <t>F-02, F-07 (en contra: E3, E4)</t>
   </si>
   <si>
     <t>N-01 (parte)</t>
@@ -7088,7 +7094,7 @@
     <t>—</t>
   </si>
   <si>
-    <t>F-03 (Reglamento 178/2002), F-04</t>
+    <t>F-03 (Reglamento 178/2002), F-04, F-07 (E4; E1 y E2 comparativos)</t>
   </si>
   <si>
     <t>N-04 y N-05 (parte)</t>
@@ -50614,16 +50620,16 @@
         <v>2310</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>921</v>
+        <v>2311</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>2311</v>
+        <v>2312</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>2312</v>
+        <v>2313</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>2313</v>
+        <v>2314</v>
       </c>
       <c r="I2" s="2">
         <v>21</v>
@@ -50646,16 +50652,16 @@
         <v>2310</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>921</v>
+        <v>2311</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>2314</v>
+        <v>2315</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>2312</v>
+        <v>2313</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>2312</v>
+        <v>2313</v>
       </c>
       <c r="I3" s="2">
         <v>19</v>
@@ -50678,16 +50684,16 @@
         <v>2310</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>921</v>
+        <v>2311</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>2315</v>
+        <v>2316</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>2316</v>
+        <v>2317</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>2317</v>
+        <v>2318</v>
       </c>
       <c r="I4" s="2">
         <v>162</v>
@@ -50713,13 +50719,13 @@
         <v>921</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>2318</v>
+        <v>2319</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>2316</v>
+        <v>2317</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>2319</v>
+        <v>2320</v>
       </c>
       <c r="I5" s="2">
         <v>33</v>
@@ -50742,16 +50748,16 @@
         <v>2310</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>921</v>
+        <v>2311</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>2320</v>
+        <v>2321</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>2321</v>
+        <v>2322</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>2322</v>
+        <v>2323</v>
       </c>
       <c r="I6" s="2">
         <v>8</v>
@@ -50774,16 +50780,16 @@
         <v>2310</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>921</v>
+        <v>2324</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>2323</v>
+        <v>2325</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>2324</v>
+        <v>2326</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>2325</v>
+        <v>2327</v>
       </c>
       <c r="I7" s="2">
         <v>10</v>
@@ -50803,19 +50809,19 @@
         <v>2309</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>2327</v>
+        <v>2329</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>2328</v>
+        <v>2330</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="I8" s="2">
         <v>11</v>
@@ -50838,16 +50844,16 @@
         <v>2310</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>921</v>
+        <v>2311</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>2330</v>
+        <v>2332</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>2331</v>
+        <v>2333</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="I9" s="2">
         <v>36</v>
@@ -50867,19 +50873,19 @@
         <v>2309</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>2333</v>
+        <v>2335</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>2334</v>
+        <v>2336</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="I10" s="2">
         <v>14</v>
@@ -50899,19 +50905,19 @@
         <v>2309</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>2335</v>
+        <v>2337</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>2328</v>
+        <v>2330</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="I11" s="2">
         <v>35</v>
@@ -50928,22 +50934,22 @@
         <v>115</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>2336</v>
+        <v>2338</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>2337</v>
+        <v>2339</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>2328</v>
+        <v>2330</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="I12" s="2">
         <v>61</v>
@@ -50969,13 +50975,13 @@
         <v>921</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>2338</v>
+        <v>2340</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>2339</v>
+        <v>2341</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="I13" s="2">
         <v>34</v>
@@ -50992,7 +50998,7 @@
         <v>405</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>2340</v>
+        <v>2342</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>2310</v>
@@ -51001,13 +51007,13 @@
         <v>921</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>2341</v>
+        <v>2343</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>2342</v>
+        <v>2344</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>2343</v>
+        <v>2345</v>
       </c>
       <c r="I14" s="2">
         <v>15</v>
@@ -51024,7 +51030,7 @@
         <v>316</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>2340</v>
+        <v>2342</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>2310</v>
@@ -51033,13 +51039,13 @@
         <v>921</v>
       </c>
       <c r="F15" s="2" t="s">
+        <v>2346</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>2344</v>
       </c>
-      <c r="G15" s="2" t="s">
-        <v>2342</v>
-      </c>
       <c r="H15" s="2" t="s">
-        <v>2345</v>
+        <v>2347</v>
       </c>
       <c r="I15" s="2">
         <v>16</v>
@@ -51056,7 +51062,7 @@
         <v>837</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>2340</v>
+        <v>2342</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>2310</v>
@@ -51065,13 +51071,13 @@
         <v>921</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>2346</v>
+        <v>2348</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>2347</v>
+        <v>2349</v>
       </c>
       <c r="I16" s="2">
         <v>1</v>
@@ -51088,7 +51094,7 @@
         <v>1155</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>2340</v>
+        <v>2342</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>2310</v>
@@ -51097,13 +51103,13 @@
         <v>921</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>2348</v>
+        <v>2350</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>2349</v>
+        <v>2351</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>2350</v>
+        <v>2352</v>
       </c>
       <c r="I17" s="2">
         <v>13</v>
@@ -51120,7 +51126,7 @@
         <v>418</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>2340</v>
+        <v>2342</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>2310</v>
@@ -51129,13 +51135,13 @@
         <v>921</v>
       </c>
       <c r="F18" s="2" t="s">
+        <v>2353</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>2351</v>
       </c>
-      <c r="G18" s="2" t="s">
-        <v>2349</v>
-      </c>
       <c r="H18" s="2" t="s">
-        <v>2352</v>
+        <v>2354</v>
       </c>
       <c r="I18" s="2">
         <v>11</v>
@@ -51152,7 +51158,7 @@
         <v>99</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>2340</v>
+        <v>2342</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>2310</v>
@@ -51161,13 +51167,13 @@
         <v>921</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>2353</v>
+        <v>2355</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>2349</v>
+        <v>2351</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>2354</v>
+        <v>2356</v>
       </c>
       <c r="I19" s="2">
         <v>24</v>
@@ -51184,22 +51190,22 @@
         <v>172</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>2355</v>
+        <v>2357</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>2356</v>
+        <v>2358</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>2357</v>
+        <v>2359</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="I20" s="2">
         <v>9</v>
@@ -51216,7 +51222,7 @@
         <v>1213</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>2358</v>
+        <v>2360</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>2310</v>
@@ -51225,13 +51231,13 @@
         <v>921</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>2348</v>
+        <v>2350</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>2359</v>
+        <v>2361</v>
       </c>
       <c r="I21" s="2">
         <v>6</v>
@@ -51248,22 +51254,22 @@
         <v>1268</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>2358</v>
+        <v>2360</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>2360</v>
+        <v>2362</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>2361</v>
+        <v>2363</v>
       </c>
       <c r="I22" s="2">
         <v>4</v>
@@ -51280,7 +51286,7 @@
         <v>1179</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>2358</v>
+        <v>2360</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>2310</v>
@@ -51289,13 +51295,13 @@
         <v>921</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>2348</v>
+        <v>2350</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>2362</v>
+        <v>2364</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>2363</v>
+        <v>2365</v>
       </c>
       <c r="I23" s="2">
         <v>16</v>
@@ -51330,7 +51336,7 @@
         <v>33</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2364</v>
+        <v>2366</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>41</v>
@@ -51351,36 +51357,36 @@
         <v>46</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>2365</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="2" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>2366</v>
+        <v>2368</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>2368</v>
+        <v>2370</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>2369</v>
+        <v>2371</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>2370</v>
+        <v>2372</v>
       </c>
       <c r="F2" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G2" s="15" t="s">
-        <v>2371</v>
+        <v>2373</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>2372</v>
+        <v>2374</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>2373</v>
+        <v>2375</v>
       </c>
       <c r="J2" s="2">
         <v>35</v>
@@ -51388,13 +51394,13 @@
     </row>
     <row r="3" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>2374</v>
+        <v>2376</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>2375</v>
+        <v>2377</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>63</v>
@@ -51420,13 +51426,13 @@
     </row>
     <row r="4" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>2376</v>
+        <v>2378</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>2377</v>
+        <v>2379</v>
       </c>
       <c r="D4" s="10" t="s">
         <v>63</v>
@@ -51452,19 +51458,19 @@
     </row>
     <row r="5" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>2378</v>
+        <v>2380</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>2379</v>
+        <v>2381</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>2380</v>
+        <v>2382</v>
       </c>
       <c r="F5" s="10" t="s">
         <v>63</v>
@@ -51484,16 +51490,16 @@
     </row>
     <row r="6" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>2381</v>
+        <v>2383</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>2382</v>
+        <v>2384</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>2383</v>
+        <v>2385</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>63</v>
@@ -51516,16 +51522,16 @@
     </row>
     <row r="7" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>2384</v>
+        <v>2386</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>2385</v>
+        <v>2387</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>2386</v>
+        <v>2388</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>63</v>
@@ -51534,10 +51540,10 @@
         <v>63</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>2387</v>
+        <v>2389</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>2388</v>
+        <v>2390</v>
       </c>
       <c r="I7" s="10" t="s">
         <v>63</v>
@@ -51548,19 +51554,19 @@
     </row>
     <row r="8" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>2389</v>
+        <v>2391</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>2390</v>
+        <v>2392</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>2391</v>
+        <v>2393</v>
       </c>
       <c r="F8" s="10" t="s">
         <v>63</v>
@@ -51580,19 +51586,19 @@
     </row>
     <row r="9" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>2392</v>
+        <v>2394</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>2393</v>
+        <v>2395</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>2394</v>
+        <v>2396</v>
       </c>
       <c r="F9" s="10" t="s">
         <v>63</v>
@@ -51612,16 +51618,16 @@
     </row>
     <row r="10" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>2395</v>
+        <v>2397</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>2397</v>
+        <v>2399</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>63</v>
@@ -51636,7 +51642,7 @@
         <v>63</v>
       </c>
       <c r="I10" s="15" t="s">
-        <v>2398</v>
+        <v>2400</v>
       </c>
       <c r="J10" s="2">
         <v>6</v>
@@ -51644,16 +51650,16 @@
     </row>
     <row r="11" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>2399</v>
+        <v>2401</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>2400</v>
+        <v>2402</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>2401</v>
+        <v>2403</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>63</v>
@@ -51662,7 +51668,7 @@
         <v>63</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>2402</v>
+        <v>2404</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>63</v>
@@ -51676,13 +51682,13 @@
     </row>
     <row r="12" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>2403</v>
+        <v>2405</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>2404</v>
+        <v>2406</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>63</v>
@@ -51694,7 +51700,7 @@
         <v>63</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>2405</v>
+        <v>2407</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>63</v>
@@ -51708,22 +51714,22 @@
     </row>
     <row r="13" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>2406</v>
+        <v>2408</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>2408</v>
+        <v>2410</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>2409</v>
+        <v>2411</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>2410</v>
+        <v>2412</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>2411</v>
+        <v>2413</v>
       </c>
       <c r="G13" s="10" t="s">
         <v>63</v>
@@ -51732,7 +51738,7 @@
         <v>63</v>
       </c>
       <c r="I13" s="15" t="s">
-        <v>2412</v>
+        <v>2414</v>
       </c>
       <c r="J13" s="2">
         <v>4</v>
@@ -51740,16 +51746,16 @@
     </row>
     <row r="14" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>2413</v>
+        <v>2415</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>2414</v>
+        <v>2416</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>2415</v>
+        <v>2417</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>63</v>
@@ -51764,7 +51770,7 @@
         <v>63</v>
       </c>
       <c r="I14" s="15" t="s">
-        <v>2416</v>
+        <v>2418</v>
       </c>
       <c r="J14" s="2">
         <v>9</v>
@@ -51772,31 +51778,31 @@
     </row>
     <row r="15" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>2417</v>
+        <v>2419</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>2418</v>
+        <v>2420</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>2419</v>
+        <v>2421</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>63</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>2420</v>
+        <v>2422</v>
       </c>
       <c r="G15" s="10" t="s">
         <v>63</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>2421</v>
+        <v>2423</v>
       </c>
       <c r="I15" s="15" t="s">
-        <v>2422</v>
+        <v>2424</v>
       </c>
       <c r="J15" s="2">
         <v>6</v>
@@ -51804,13 +51810,13 @@
     </row>
     <row r="16" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>2423</v>
+        <v>2425</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>2424</v>
+        <v>2426</v>
       </c>
       <c r="D16" s="10" t="s">
         <v>63</v>
@@ -51828,7 +51834,7 @@
         <v>63</v>
       </c>
       <c r="I16" s="15" t="s">
-        <v>2425</v>
+        <v>2427</v>
       </c>
       <c r="J16" s="2">
         <v>21</v>
@@ -51836,13 +51842,13 @@
     </row>
     <row r="17" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>2426</v>
+        <v>2428</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>2427</v>
+        <v>2429</v>
       </c>
       <c r="D17" s="10" t="s">
         <v>63</v>
@@ -51857,10 +51863,10 @@
         <v>63</v>
       </c>
       <c r="H17" s="15" t="s">
-        <v>2428</v>
+        <v>2430</v>
       </c>
       <c r="I17" s="15" t="s">
-        <v>2429</v>
+        <v>2431</v>
       </c>
       <c r="J17" s="2">
         <v>8</v>
@@ -51868,16 +51874,16 @@
     </row>
     <row r="18" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>2430</v>
+        <v>2432</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>2431</v>
+        <v>2433</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>2432</v>
+        <v>2434</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>63</v>
@@ -51886,13 +51892,13 @@
         <v>63</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>2433</v>
+        <v>2435</v>
       </c>
       <c r="H18" s="15" t="s">
-        <v>2434</v>
+        <v>2436</v>
       </c>
       <c r="I18" s="15" t="s">
-        <v>2435</v>
+        <v>2437</v>
       </c>
       <c r="J18" s="2">
         <v>5</v>
@@ -51900,16 +51906,16 @@
     </row>
     <row r="19" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>2436</v>
+        <v>2438</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>2437</v>
+        <v>2439</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>2438</v>
+        <v>2440</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>63</v>
@@ -51924,7 +51930,7 @@
         <v>63</v>
       </c>
       <c r="I19" s="15" t="s">
-        <v>2439</v>
+        <v>2441</v>
       </c>
       <c r="J19" s="2">
         <v>4</v>
@@ -51932,13 +51938,13 @@
     </row>
     <row r="20" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>2440</v>
+        <v>2442</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>2441</v>
+        <v>2443</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>63</v>
@@ -51956,7 +51962,7 @@
         <v>63</v>
       </c>
       <c r="I20" s="15" t="s">
-        <v>2442</v>
+        <v>2444</v>
       </c>
       <c r="J20" s="2">
         <v>2</v>
@@ -51964,16 +51970,16 @@
     </row>
     <row r="21" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>2443</v>
+        <v>2445</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>2444</v>
+        <v>2446</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>2445</v>
+        <v>2447</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>63</v>
@@ -51985,7 +51991,7 @@
         <v>63</v>
       </c>
       <c r="H21" s="16" t="s">
-        <v>2446</v>
+        <v>2448</v>
       </c>
       <c r="I21" s="10" t="s">
         <v>63</v>
@@ -51996,13 +52002,13 @@
     </row>
     <row r="22" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>2447</v>
+        <v>2449</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>2448</v>
+        <v>2450</v>
       </c>
       <c r="D22" s="10" t="s">
         <v>63</v>
@@ -52014,10 +52020,10 @@
         <v>63</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>2449</v>
+        <v>2451</v>
       </c>
       <c r="H22" s="15" t="s">
-        <v>2450</v>
+        <v>2452</v>
       </c>
       <c r="I22" s="10" t="s">
         <v>63</v>
@@ -52028,16 +52034,16 @@
     </row>
     <row r="23" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>2451</v>
+        <v>2453</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>2452</v>
+        <v>2454</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>2453</v>
+        <v>2455</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>63</v>
@@ -52060,13 +52066,13 @@
     </row>
     <row r="24" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>2454</v>
+        <v>2456</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>2455</v>
+        <v>2457</v>
       </c>
       <c r="D24" s="10" t="s">
         <v>63</v>
@@ -52084,7 +52090,7 @@
         <v>63</v>
       </c>
       <c r="I24" s="15" t="s">
-        <v>2456</v>
+        <v>2458</v>
       </c>
       <c r="J24" s="2">
         <v>0</v>
@@ -52092,31 +52098,31 @@
     </row>
     <row r="25" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>2457</v>
+        <v>2459</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>2458</v>
+        <v>2460</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>2459</v>
+        <v>2461</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>2432</v>
+        <v>2434</v>
       </c>
       <c r="E25" s="16" t="s">
-        <v>2460</v>
+        <v>2462</v>
       </c>
       <c r="F25" s="16" t="s">
-        <v>2461</v>
+        <v>2463</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>2433</v>
+        <v>2435</v>
       </c>
       <c r="H25" s="15" t="s">
-        <v>2462</v>
+        <v>2464</v>
       </c>
       <c r="I25" s="15" t="s">
-        <v>2463</v>
+        <v>2465</v>
       </c>
       <c r="J25" s="2">
         <v>25</v>
@@ -52124,16 +52130,16 @@
     </row>
     <row r="26" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>2464</v>
+        <v>2466</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>2458</v>
+        <v>2460</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>2465</v>
+        <v>2467</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>2466</v>
+        <v>2468</v>
       </c>
       <c r="E26" s="10" t="s">
         <v>63</v>
@@ -52156,19 +52162,19 @@
     </row>
     <row r="27" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>2467</v>
+        <v>2469</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>2458</v>
+        <v>2460</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>2468</v>
+        <v>2470</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>2469</v>
+        <v>2471</v>
       </c>
       <c r="E27" s="16" t="s">
-        <v>2470</v>
+        <v>2472</v>
       </c>
       <c r="F27" s="10" t="s">
         <v>63</v>
@@ -52177,7 +52183,7 @@
         <v>63</v>
       </c>
       <c r="H27" s="15" t="s">
-        <v>2471</v>
+        <v>2473</v>
       </c>
       <c r="I27" s="10" t="s">
         <v>63</v>
@@ -52188,19 +52194,19 @@
     </row>
     <row r="28" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>2472</v>
+        <v>2474</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>2458</v>
+        <v>2460</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>2473</v>
+        <v>2475</v>
       </c>
       <c r="D28" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>2474</v>
+        <v>2476</v>
       </c>
       <c r="F28" s="10" t="s">
         <v>63</v>
@@ -52220,16 +52226,16 @@
     </row>
     <row r="29" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>2475</v>
+        <v>2477</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>2458</v>
+        <v>2460</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>2476</v>
+        <v>2478</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>2477</v>
+        <v>2479</v>
       </c>
       <c r="E29" s="10" t="s">
         <v>63</v>
@@ -52252,16 +52258,16 @@
     </row>
     <row r="30" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>2478</v>
+        <v>2480</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>2458</v>
+        <v>2460</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>2479</v>
+        <v>2481</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>2480</v>
+        <v>2482</v>
       </c>
       <c r="E30" s="10" t="s">
         <v>63</v>
@@ -52276,7 +52282,7 @@
         <v>63</v>
       </c>
       <c r="I30" s="15" t="s">
-        <v>2481</v>
+        <v>2483</v>
       </c>
       <c r="J30" s="2">
         <v>12</v>
@@ -52284,31 +52290,31 @@
     </row>
     <row r="31" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>2482</v>
+        <v>2484</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>2484</v>
+        <v>2486</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>2485</v>
+        <v>2487</v>
       </c>
       <c r="E31" s="15" t="s">
-        <v>2486</v>
+        <v>2488</v>
       </c>
       <c r="F31" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G31" s="15" t="s">
-        <v>2487</v>
+        <v>2489</v>
       </c>
       <c r="H31" s="15" t="s">
-        <v>2488</v>
+        <v>2490</v>
       </c>
       <c r="I31" s="15" t="s">
-        <v>2489</v>
+        <v>2491</v>
       </c>
       <c r="J31" s="2">
         <v>5</v>
@@ -52316,19 +52322,19 @@
     </row>
     <row r="32" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>2490</v>
+        <v>2492</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>2491</v>
+        <v>2493</v>
       </c>
       <c r="D32" s="16" t="s">
-        <v>2492</v>
+        <v>2494</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>2493</v>
+        <v>2495</v>
       </c>
       <c r="F32" s="10" t="s">
         <v>63</v>
@@ -52337,10 +52343,10 @@
         <v>63</v>
       </c>
       <c r="H32" s="15" t="s">
-        <v>2494</v>
+        <v>2496</v>
       </c>
       <c r="I32" s="15" t="s">
-        <v>2495</v>
+        <v>2497</v>
       </c>
       <c r="J32" s="2">
         <v>4</v>
@@ -52348,25 +52354,25 @@
     </row>
     <row r="33" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>2496</v>
+        <v>2498</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>2497</v>
+        <v>2499</v>
       </c>
       <c r="D33" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E33" s="15" t="s">
-        <v>2498</v>
+        <v>2500</v>
       </c>
       <c r="F33" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G33" s="15" t="s">
-        <v>2499</v>
+        <v>2501</v>
       </c>
       <c r="H33" s="10" t="s">
         <v>63</v>
@@ -52380,19 +52386,19 @@
     </row>
     <row r="34" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>2500</v>
+        <v>2502</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>2501</v>
+        <v>2503</v>
       </c>
       <c r="D34" s="16" t="s">
-        <v>2492</v>
+        <v>2494</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>2502</v>
+        <v>2504</v>
       </c>
       <c r="F34" s="10" t="s">
         <v>63</v>
@@ -52404,7 +52410,7 @@
         <v>63</v>
       </c>
       <c r="I34" s="15" t="s">
-        <v>2503</v>
+        <v>2505</v>
       </c>
       <c r="J34" s="2">
         <v>0</v>
@@ -52412,16 +52418,16 @@
     </row>
     <row r="35" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>2504</v>
+        <v>2506</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>2505</v>
+        <v>2507</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>2506</v>
+        <v>2508</v>
       </c>
       <c r="E35" s="10" t="s">
         <v>63</v>
@@ -52444,19 +52450,19 @@
     </row>
     <row r="36" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>2507</v>
+        <v>2509</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>2508</v>
+        <v>2510</v>
       </c>
       <c r="D36" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E36" s="15" t="s">
-        <v>2509</v>
+        <v>2511</v>
       </c>
       <c r="F36" s="10" t="s">
         <v>63</v>
@@ -52476,19 +52482,19 @@
     </row>
     <row r="37" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>2510</v>
+        <v>2512</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>2511</v>
+        <v>2513</v>
       </c>
       <c r="D37" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E37" s="15" t="s">
-        <v>2512</v>
+        <v>2514</v>
       </c>
       <c r="F37" s="10" t="s">
         <v>63</v>
@@ -52508,13 +52514,13 @@
     </row>
     <row r="38" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>2513</v>
+        <v>2515</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>2514</v>
+        <v>2516</v>
       </c>
       <c r="D38" s="10" t="s">
         <v>63</v>
@@ -52532,7 +52538,7 @@
         <v>63</v>
       </c>
       <c r="I38" s="15" t="s">
-        <v>2515</v>
+        <v>2517</v>
       </c>
       <c r="J38" s="2">
         <v>0</v>
@@ -52540,13 +52546,13 @@
     </row>
     <row r="39" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>2516</v>
+        <v>2518</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>2517</v>
+        <v>2519</v>
       </c>
       <c r="D39" s="10" t="s">
         <v>63</v>
@@ -52564,7 +52570,7 @@
         <v>63</v>
       </c>
       <c r="I39" s="15" t="s">
-        <v>2518</v>
+        <v>2520</v>
       </c>
       <c r="J39" s="2">
         <v>12</v>
@@ -52572,13 +52578,13 @@
     </row>
     <row r="40" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>2519</v>
+        <v>2521</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>2520</v>
+        <v>2522</v>
       </c>
       <c r="D40" s="10" t="s">
         <v>63</v>
@@ -52596,7 +52602,7 @@
         <v>63</v>
       </c>
       <c r="I40" s="15" t="s">
-        <v>2521</v>
+        <v>2523</v>
       </c>
       <c r="J40" s="2">
         <v>0</v>
@@ -52604,31 +52610,31 @@
     </row>
     <row r="41" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>2522</v>
+        <v>2524</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>2523</v>
+        <v>2525</v>
       </c>
       <c r="D41" s="15" t="s">
-        <v>2524</v>
+        <v>2526</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>2525</v>
+        <v>2527</v>
       </c>
       <c r="F41" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G41" s="15" t="s">
-        <v>2526</v>
+        <v>2528</v>
       </c>
       <c r="H41" s="10" t="s">
         <v>63</v>
       </c>
       <c r="I41" s="15" t="s">
-        <v>2527</v>
+        <v>2529</v>
       </c>
       <c r="J41" s="2">
         <v>1</v>
@@ -52636,19 +52642,19 @@
     </row>
     <row r="42" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>2528</v>
+        <v>2530</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>2529</v>
+        <v>2531</v>
       </c>
       <c r="D42" s="15" t="s">
-        <v>2530</v>
+        <v>2532</v>
       </c>
       <c r="E42" s="15" t="s">
-        <v>2531</v>
+        <v>2533</v>
       </c>
       <c r="F42" s="10" t="s">
         <v>63</v>
@@ -52668,31 +52674,31 @@
     </row>
     <row r="43" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>2532</v>
+        <v>2534</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>2533</v>
+        <v>2535</v>
       </c>
       <c r="D43" s="15" t="s">
-        <v>2534</v>
+        <v>2536</v>
       </c>
       <c r="E43" s="15" t="s">
-        <v>2535</v>
+        <v>2537</v>
       </c>
       <c r="F43" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G43" s="15" t="s">
-        <v>2536</v>
+        <v>2538</v>
       </c>
       <c r="H43" s="15" t="s">
-        <v>2537</v>
+        <v>2539</v>
       </c>
       <c r="I43" s="15" t="s">
-        <v>2538</v>
+        <v>2540</v>
       </c>
       <c r="J43" s="2">
         <v>2</v>
@@ -52700,16 +52706,16 @@
     </row>
     <row r="44" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>2539</v>
+        <v>2541</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>2540</v>
+        <v>2542</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>2541</v>
+        <v>2543</v>
       </c>
       <c r="E44" s="10" t="s">
         <v>63</v>
@@ -52718,13 +52724,13 @@
         <v>63</v>
       </c>
       <c r="G44" s="15" t="s">
-        <v>2542</v>
+        <v>2544</v>
       </c>
       <c r="H44" s="10" t="s">
         <v>63</v>
       </c>
       <c r="I44" s="15" t="s">
-        <v>2543</v>
+        <v>2545</v>
       </c>
       <c r="J44" s="2">
         <v>4</v>
@@ -52732,31 +52738,31 @@
     </row>
     <row r="45" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>2544</v>
+        <v>2546</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>2545</v>
+        <v>2547</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>2546</v>
+        <v>2548</v>
       </c>
       <c r="D45" s="15" t="s">
-        <v>2547</v>
+        <v>2549</v>
       </c>
       <c r="E45" s="15" t="s">
-        <v>2548</v>
+        <v>2550</v>
       </c>
       <c r="F45" s="16" t="s">
-        <v>2549</v>
+        <v>2551</v>
       </c>
       <c r="G45" s="15" t="s">
-        <v>2550</v>
+        <v>2552</v>
       </c>
       <c r="H45" s="15" t="s">
-        <v>2551</v>
+        <v>2553</v>
       </c>
       <c r="I45" s="9" t="s">
-        <v>2552</v>
+        <v>2554</v>
       </c>
       <c r="J45" s="2">
         <v>3</v>
@@ -52764,31 +52770,31 @@
     </row>
     <row r="46" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>2553</v>
+        <v>2555</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>2545</v>
+        <v>2547</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>2554</v>
+        <v>2556</v>
       </c>
       <c r="D46" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E46" s="15" t="s">
-        <v>2555</v>
+        <v>2557</v>
       </c>
       <c r="F46" s="15" t="s">
-        <v>2556</v>
+        <v>2558</v>
       </c>
       <c r="G46" s="10" t="s">
         <v>63</v>
       </c>
       <c r="H46" s="15" t="s">
-        <v>2557</v>
+        <v>2559</v>
       </c>
       <c r="I46" s="15" t="s">
-        <v>2558</v>
+        <v>2560</v>
       </c>
       <c r="J46" s="2">
         <v>3</v>
@@ -52796,25 +52802,25 @@
     </row>
     <row r="47" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>2559</v>
+        <v>2561</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>2545</v>
+        <v>2547</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>2560</v>
+        <v>2562</v>
       </c>
       <c r="D47" s="15" t="s">
-        <v>2561</v>
+        <v>2563</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>2562</v>
+        <v>2564</v>
       </c>
       <c r="F47" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G47" s="15" t="s">
-        <v>2563</v>
+        <v>2565</v>
       </c>
       <c r="H47" s="10" t="s">
         <v>63</v>
@@ -52828,13 +52834,13 @@
     </row>
     <row r="48" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>2564</v>
+        <v>2566</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>2545</v>
+        <v>2547</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>2565</v>
+        <v>2567</v>
       </c>
       <c r="D48" s="10" t="s">
         <v>63</v>
@@ -52846,10 +52852,10 @@
         <v>63</v>
       </c>
       <c r="G48" s="15" t="s">
-        <v>2566</v>
+        <v>2568</v>
       </c>
       <c r="H48" s="15" t="s">
-        <v>2567</v>
+        <v>2569</v>
       </c>
       <c r="I48" s="10" t="s">
         <v>63</v>
@@ -52860,13 +52866,13 @@
     </row>
     <row r="49" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>2568</v>
+        <v>2570</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>2545</v>
+        <v>2547</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>2569</v>
+        <v>2571</v>
       </c>
       <c r="D49" s="10" t="s">
         <v>63</v>
@@ -52881,10 +52887,10 @@
         <v>63</v>
       </c>
       <c r="H49" s="15" t="s">
-        <v>2570</v>
+        <v>2572</v>
       </c>
       <c r="I49" s="15" t="s">
-        <v>2571</v>
+        <v>2573</v>
       </c>
       <c r="J49" s="2">
         <v>15</v>
@@ -52892,13 +52898,13 @@
     </row>
     <row r="50" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>2572</v>
+        <v>2574</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>2573</v>
+        <v>2575</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>2574</v>
+        <v>2576</v>
       </c>
       <c r="D50" s="10" t="s">
         <v>63</v>
@@ -52913,7 +52919,7 @@
         <v>63</v>
       </c>
       <c r="H50" s="15" t="s">
-        <v>2575</v>
+        <v>2577</v>
       </c>
       <c r="I50" s="10" t="s">
         <v>63</v>
@@ -52924,13 +52930,13 @@
     </row>
     <row r="51" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>2576</v>
+        <v>2578</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>2545</v>
+        <v>2547</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>2577</v>
+        <v>2579</v>
       </c>
       <c r="D51" s="10" t="s">
         <v>63</v>
@@ -52945,7 +52951,7 @@
         <v>63</v>
       </c>
       <c r="H51" s="16" t="s">
-        <v>2578</v>
+        <v>2580</v>
       </c>
       <c r="I51" s="10" t="s">
         <v>63</v>
@@ -52956,13 +52962,13 @@
     </row>
     <row r="52" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>2579</v>
+        <v>2581</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>2573</v>
+        <v>2575</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>2580</v>
+        <v>2582</v>
       </c>
       <c r="D52" s="10" t="s">
         <v>63</v>
@@ -52977,7 +52983,7 @@
         <v>63</v>
       </c>
       <c r="H52" s="15" t="s">
-        <v>2581</v>
+        <v>2583</v>
       </c>
       <c r="I52" s="10" t="s">
         <v>63</v>
@@ -52988,13 +52994,13 @@
     </row>
     <row r="53" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>2582</v>
+        <v>2584</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>2545</v>
+        <v>2547</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>2583</v>
+        <v>2585</v>
       </c>
       <c r="D53" s="10" t="s">
         <v>63</v>
@@ -53009,7 +53015,7 @@
         <v>63</v>
       </c>
       <c r="H53" s="15" t="s">
-        <v>2584</v>
+        <v>2586</v>
       </c>
       <c r="I53" s="10" t="s">
         <v>63</v>
@@ -53020,19 +53026,19 @@
     </row>
     <row r="54" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>2585</v>
+        <v>2587</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>2586</v>
+        <v>2588</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>2587</v>
+        <v>2589</v>
       </c>
       <c r="D54" s="15" t="s">
-        <v>2588</v>
+        <v>2590</v>
       </c>
       <c r="E54" s="15" t="s">
-        <v>2589</v>
+        <v>2591</v>
       </c>
       <c r="F54" s="10" t="s">
         <v>63</v>
@@ -53052,19 +53058,19 @@
     </row>
     <row r="55" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>2590</v>
+        <v>2592</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>2586</v>
+        <v>2588</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>2591</v>
+        <v>2593</v>
       </c>
       <c r="D55" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E55" s="15" t="s">
-        <v>2592</v>
+        <v>2594</v>
       </c>
       <c r="F55" s="10" t="s">
         <v>63</v>
@@ -53084,19 +53090,19 @@
     </row>
     <row r="56" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>2593</v>
+        <v>2595</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>2586</v>
+        <v>2588</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>2594</v>
+        <v>2596</v>
       </c>
       <c r="D56" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E56" s="15" t="s">
-        <v>2595</v>
+        <v>2597</v>
       </c>
       <c r="F56" s="10" t="s">
         <v>63</v>
@@ -53116,28 +53122,28 @@
     </row>
     <row r="57" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>2596</v>
+        <v>2598</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>2597</v>
+        <v>2599</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>2598</v>
+        <v>2600</v>
       </c>
       <c r="D57" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E57" s="15" t="s">
-        <v>2599</v>
+        <v>2601</v>
       </c>
       <c r="F57" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G57" s="15" t="s">
-        <v>2600</v>
+        <v>2602</v>
       </c>
       <c r="H57" s="15" t="s">
-        <v>2601</v>
+        <v>2603</v>
       </c>
       <c r="I57" s="10" t="s">
         <v>63</v>
@@ -53148,13 +53154,13 @@
     </row>
     <row r="58" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>2602</v>
+        <v>2604</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>2597</v>
+        <v>2599</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>2603</v>
+        <v>2605</v>
       </c>
       <c r="D58" s="10" t="s">
         <v>63</v>
@@ -53169,7 +53175,7 @@
         <v>63</v>
       </c>
       <c r="H58" s="15" t="s">
-        <v>2604</v>
+        <v>2606</v>
       </c>
       <c r="I58" s="10" t="s">
         <v>63</v>
@@ -53180,19 +53186,19 @@
     </row>
     <row r="59" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>2605</v>
+        <v>2607</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>2597</v>
+        <v>2599</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>2606</v>
+        <v>2608</v>
       </c>
       <c r="D59" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>2607</v>
+        <v>2609</v>
       </c>
       <c r="F59" s="10" t="s">
         <v>63</v>
@@ -53201,7 +53207,7 @@
         <v>63</v>
       </c>
       <c r="H59" s="15" t="s">
-        <v>2608</v>
+        <v>2610</v>
       </c>
       <c r="I59" s="10" t="s">
         <v>63</v>
@@ -53212,19 +53218,19 @@
     </row>
     <row r="60" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>2609</v>
+        <v>2611</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>2597</v>
+        <v>2599</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>2610</v>
+        <v>2612</v>
       </c>
       <c r="D60" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E60" s="15" t="s">
-        <v>2611</v>
+        <v>2613</v>
       </c>
       <c r="F60" s="10" t="s">
         <v>63</v>
@@ -53233,7 +53239,7 @@
         <v>63</v>
       </c>
       <c r="H60" s="15" t="s">
-        <v>2612</v>
+        <v>2614</v>
       </c>
       <c r="I60" s="10" t="s">
         <v>63</v>
@@ -53244,19 +53250,19 @@
     </row>
     <row r="61" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>2613</v>
+        <v>2615</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>2597</v>
+        <v>2599</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>2614</v>
+        <v>2616</v>
       </c>
       <c r="D61" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E61" s="15" t="s">
-        <v>2615</v>
+        <v>2617</v>
       </c>
       <c r="F61" s="10" t="s">
         <v>63</v>
@@ -53276,25 +53282,25 @@
     </row>
     <row r="62" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>2616</v>
+        <v>2618</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>2617</v>
+        <v>2619</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>2618</v>
+        <v>2620</v>
       </c>
       <c r="D62" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E62" s="9" t="s">
-        <v>2619</v>
+        <v>2621</v>
       </c>
       <c r="F62" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G62" s="9" t="s">
-        <v>2620</v>
+        <v>2622</v>
       </c>
       <c r="H62" s="10" t="s">
         <v>63</v>
@@ -53308,31 +53314,31 @@
     </row>
     <row r="63" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>2621</v>
+        <v>2623</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>2622</v>
+        <v>2624</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>2623</v>
+        <v>2625</v>
       </c>
       <c r="D63" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E63" s="15" t="s">
-        <v>2624</v>
+        <v>2626</v>
       </c>
       <c r="F63" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G63" s="15" t="s">
-        <v>2625</v>
+        <v>2627</v>
       </c>
       <c r="H63" s="10" t="s">
         <v>63</v>
       </c>
       <c r="I63" s="15" t="s">
-        <v>2626</v>
+        <v>2628</v>
       </c>
       <c r="J63" s="2">
         <v>4</v>
@@ -53340,13 +53346,13 @@
     </row>
     <row r="64" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>2627</v>
+        <v>2629</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>2622</v>
+        <v>2624</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>2628</v>
+        <v>2630</v>
       </c>
       <c r="D64" s="10" t="s">
         <v>63</v>
@@ -53358,7 +53364,7 @@
         <v>63</v>
       </c>
       <c r="G64" s="15" t="s">
-        <v>2629</v>
+        <v>2631</v>
       </c>
       <c r="H64" s="10" t="s">
         <v>63</v>
@@ -53372,25 +53378,25 @@
     </row>
     <row r="65" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>2630</v>
+        <v>2632</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>2622</v>
+        <v>2624</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>2631</v>
+        <v>2633</v>
       </c>
       <c r="D65" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E65" s="15" t="s">
-        <v>2632</v>
+        <v>2634</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G65" s="15" t="s">
-        <v>2633</v>
+        <v>2635</v>
       </c>
       <c r="H65" s="10" t="s">
         <v>63</v>
@@ -53404,13 +53410,13 @@
     </row>
     <row r="66" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>2634</v>
+        <v>2636</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>2635</v>
+        <v>2637</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>2636</v>
+        <v>2638</v>
       </c>
       <c r="D66" s="10" t="s">
         <v>63</v>
@@ -53422,7 +53428,7 @@
         <v>63</v>
       </c>
       <c r="G66" s="15" t="s">
-        <v>2637</v>
+        <v>2639</v>
       </c>
       <c r="H66" s="10" t="s">
         <v>63</v>
@@ -53436,19 +53442,19 @@
     </row>
     <row r="67" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>2638</v>
+        <v>2640</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>2635</v>
+        <v>2637</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>2639</v>
+        <v>2641</v>
       </c>
       <c r="D67" s="16" t="s">
-        <v>2640</v>
+        <v>2642</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>2641</v>
+        <v>2643</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>63</v>
@@ -53468,13 +53474,13 @@
     </row>
     <row r="68" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>2642</v>
+        <v>2644</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>2635</v>
+        <v>2637</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>2643</v>
+        <v>2645</v>
       </c>
       <c r="D68" s="10" t="s">
         <v>63</v>
@@ -53483,7 +53489,7 @@
         <v>63</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>2644</v>
+        <v>2646</v>
       </c>
       <c r="G68" s="10" t="s">
         <v>63</v>
@@ -53500,13 +53506,13 @@
     </row>
     <row r="69" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>2645</v>
+        <v>2647</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>2646</v>
+        <v>2648</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>2647</v>
+        <v>2649</v>
       </c>
       <c r="D69" s="10" t="s">
         <v>63</v>
@@ -53521,7 +53527,7 @@
         <v>63</v>
       </c>
       <c r="H69" s="9" t="s">
-        <v>2648</v>
+        <v>2650</v>
       </c>
       <c r="I69" s="10" t="s">
         <v>63</v>
@@ -53532,13 +53538,13 @@
     </row>
     <row r="70" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>2649</v>
+        <v>2651</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>2646</v>
+        <v>2648</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>2650</v>
+        <v>2652</v>
       </c>
       <c r="D70" s="10" t="s">
         <v>63</v>
@@ -53553,7 +53559,7 @@
         <v>63</v>
       </c>
       <c r="H70" s="15" t="s">
-        <v>2651</v>
+        <v>2653</v>
       </c>
       <c r="I70" s="10" t="s">
         <v>63</v>
@@ -53564,13 +53570,13 @@
     </row>
     <row r="71" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>2652</v>
+        <v>2654</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>2654</v>
+        <v>2656</v>
       </c>
       <c r="D71" s="10" t="s">
         <v>63</v>
@@ -53585,7 +53591,7 @@
         <v>63</v>
       </c>
       <c r="H71" s="15" t="s">
-        <v>2655</v>
+        <v>2657</v>
       </c>
       <c r="I71" s="10" t="s">
         <v>63</v>
@@ -53596,13 +53602,13 @@
     </row>
     <row r="72" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>2656</v>
+        <v>2658</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>2657</v>
+        <v>2659</v>
       </c>
       <c r="D72" s="10" t="s">
         <v>63</v>
@@ -53617,7 +53623,7 @@
         <v>63</v>
       </c>
       <c r="H72" s="15" t="s">
-        <v>2658</v>
+        <v>2660</v>
       </c>
       <c r="I72" s="10" t="s">
         <v>63</v>
@@ -53628,13 +53634,13 @@
     </row>
     <row r="73" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>2659</v>
+        <v>2661</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>2660</v>
+        <v>2662</v>
       </c>
       <c r="D73" s="10" t="s">
         <v>63</v>
@@ -53649,7 +53655,7 @@
         <v>63</v>
       </c>
       <c r="H73" s="15" t="s">
-        <v>2661</v>
+        <v>2663</v>
       </c>
       <c r="I73" s="10" t="s">
         <v>63</v>
@@ -53660,19 +53666,19 @@
     </row>
     <row r="74" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>2662</v>
+        <v>2664</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>2663</v>
+        <v>2665</v>
       </c>
       <c r="D74" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E74" s="9" t="s">
-        <v>2664</v>
+        <v>2666</v>
       </c>
       <c r="F74" s="10" t="s">
         <v>63</v>
@@ -53681,7 +53687,7 @@
         <v>63</v>
       </c>
       <c r="H74" s="15" t="s">
-        <v>2665</v>
+        <v>2667</v>
       </c>
       <c r="I74" s="10" t="s">
         <v>63</v>
@@ -53692,13 +53698,13 @@
     </row>
     <row r="75" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>2666</v>
+        <v>2668</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>2646</v>
+        <v>2648</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>2667</v>
+        <v>2669</v>
       </c>
       <c r="D75" s="10" t="s">
         <v>63</v>
@@ -53713,7 +53719,7 @@
         <v>63</v>
       </c>
       <c r="H75" s="15" t="s">
-        <v>2668</v>
+        <v>2670</v>
       </c>
       <c r="I75" s="10" t="s">
         <v>63</v>
@@ -53724,13 +53730,13 @@
     </row>
     <row r="76" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>2669</v>
+        <v>2671</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>2670</v>
+        <v>2672</v>
       </c>
       <c r="D76" s="10" t="s">
         <v>63</v>
@@ -53745,7 +53751,7 @@
         <v>63</v>
       </c>
       <c r="H76" s="9" t="s">
-        <v>2671</v>
+        <v>2673</v>
       </c>
       <c r="I76" s="10" t="s">
         <v>63</v>
@@ -53756,13 +53762,13 @@
     </row>
     <row r="77" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>2672</v>
+        <v>2674</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>2673</v>
+        <v>2675</v>
       </c>
       <c r="D77" s="10" t="s">
         <v>63</v>
@@ -53777,7 +53783,7 @@
         <v>63</v>
       </c>
       <c r="H77" s="15" t="s">
-        <v>2674</v>
+        <v>2676</v>
       </c>
       <c r="I77" s="10" t="s">
         <v>63</v>
@@ -53788,13 +53794,13 @@
     </row>
     <row r="78" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>2675</v>
+        <v>2677</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>2676</v>
+        <v>2678</v>
       </c>
       <c r="D78" s="10" t="s">
         <v>63</v>
@@ -53809,7 +53815,7 @@
         <v>63</v>
       </c>
       <c r="H78" s="15" t="s">
-        <v>2677</v>
+        <v>2679</v>
       </c>
       <c r="I78" s="10" t="s">
         <v>63</v>
@@ -53820,19 +53826,19 @@
     </row>
     <row r="79" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>2678</v>
+        <v>2680</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>2679</v>
+        <v>2681</v>
       </c>
       <c r="D79" s="16" t="s">
-        <v>2680</v>
+        <v>2682</v>
       </c>
       <c r="E79" s="15" t="s">
-        <v>2681</v>
+        <v>2683</v>
       </c>
       <c r="F79" s="10" t="s">
         <v>63</v>
@@ -53841,7 +53847,7 @@
         <v>63</v>
       </c>
       <c r="H79" s="16" t="s">
-        <v>2680</v>
+        <v>2682</v>
       </c>
       <c r="I79" s="10" t="s">
         <v>63</v>
@@ -53852,13 +53858,13 @@
     </row>
     <row r="80" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>2682</v>
+        <v>2684</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>2683</v>
+        <v>2685</v>
       </c>
       <c r="D80" s="10" t="s">
         <v>63</v>
@@ -53873,7 +53879,7 @@
         <v>63</v>
       </c>
       <c r="H80" s="15" t="s">
-        <v>2684</v>
+        <v>2686</v>
       </c>
       <c r="I80" s="10" t="s">
         <v>63</v>
@@ -53884,13 +53890,13 @@
     </row>
     <row r="81" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>2685</v>
+        <v>2687</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>2686</v>
+        <v>2688</v>
       </c>
       <c r="D81" s="10" t="s">
         <v>63</v>
@@ -53905,7 +53911,7 @@
         <v>63</v>
       </c>
       <c r="H81" s="15" t="s">
-        <v>2687</v>
+        <v>2689</v>
       </c>
       <c r="I81" s="10" t="s">
         <v>63</v>
@@ -53916,13 +53922,13 @@
     </row>
     <row r="82" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>2688</v>
+        <v>2690</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>2689</v>
+        <v>2691</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>2690</v>
+        <v>2692</v>
       </c>
       <c r="D82" s="10" t="s">
         <v>63</v>
@@ -53937,7 +53943,7 @@
         <v>63</v>
       </c>
       <c r="H82" s="15" t="s">
-        <v>2691</v>
+        <v>2693</v>
       </c>
       <c r="I82" s="10" t="s">
         <v>63</v>
@@ -53948,19 +53954,19 @@
     </row>
     <row r="83" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>2692</v>
+        <v>2694</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>2693</v>
+        <v>2695</v>
       </c>
       <c r="D83" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E83" s="15" t="s">
-        <v>2694</v>
+        <v>2696</v>
       </c>
       <c r="F83" s="10" t="s">
         <v>63</v>
@@ -53969,7 +53975,7 @@
         <v>63</v>
       </c>
       <c r="H83" s="15" t="s">
-        <v>2695</v>
+        <v>2697</v>
       </c>
       <c r="I83" s="10" t="s">
         <v>63</v>
@@ -53980,13 +53986,13 @@
     </row>
     <row r="84" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>2696</v>
+        <v>2698</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>2635</v>
+        <v>2637</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>2697</v>
+        <v>2699</v>
       </c>
       <c r="D84" s="10" t="s">
         <v>63</v>
@@ -53995,7 +54001,7 @@
         <v>63</v>
       </c>
       <c r="F84" s="15" t="s">
-        <v>2698</v>
+        <v>2700</v>
       </c>
       <c r="G84" s="10" t="s">
         <v>63</v>
@@ -54012,13 +54018,13 @@
     </row>
     <row r="85" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>2699</v>
+        <v>2701</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>2700</v>
+        <v>2702</v>
       </c>
       <c r="D85" s="10" t="s">
         <v>63</v>
@@ -54036,7 +54042,7 @@
         <v>63</v>
       </c>
       <c r="I85" s="15" t="s">
-        <v>2701</v>
+        <v>2703</v>
       </c>
       <c r="J85" s="2">
         <v>0</v>
@@ -54044,31 +54050,31 @@
     </row>
     <row r="86" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>2702</v>
+        <v>2704</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>2703</v>
+        <v>2705</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>2704</v>
+        <v>2706</v>
       </c>
       <c r="D86" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E86" s="15" t="s">
-        <v>2705</v>
+        <v>2707</v>
       </c>
       <c r="F86" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G86" s="15" t="s">
-        <v>2706</v>
+        <v>2708</v>
       </c>
       <c r="H86" s="10" t="s">
         <v>63</v>
       </c>
       <c r="I86" s="15" t="s">
-        <v>2707</v>
+        <v>2709</v>
       </c>
       <c r="J86" s="2">
         <v>3</v>
@@ -54076,19 +54082,19 @@
     </row>
     <row r="87" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>2708</v>
+        <v>2710</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>2709</v>
+        <v>2711</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>2710</v>
+        <v>2712</v>
       </c>
       <c r="D87" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E87" s="15" t="s">
-        <v>2711</v>
+        <v>2713</v>
       </c>
       <c r="F87" s="10" t="s">
         <v>63</v>
@@ -54108,16 +54114,16 @@
     </row>
     <row r="88" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>2712</v>
+        <v>2714</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>2703</v>
+        <v>2705</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>2713</v>
+        <v>2715</v>
       </c>
       <c r="D88" s="15" t="s">
-        <v>2714</v>
+        <v>2716</v>
       </c>
       <c r="E88" s="10" t="s">
         <v>63</v>
@@ -54126,7 +54132,7 @@
         <v>63</v>
       </c>
       <c r="G88" s="15" t="s">
-        <v>2715</v>
+        <v>2717</v>
       </c>
       <c r="H88" s="10" t="s">
         <v>63</v>
@@ -54140,25 +54146,25 @@
     </row>
     <row r="89" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>2716</v>
+        <v>2718</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>2703</v>
+        <v>2705</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>2717</v>
+        <v>2719</v>
       </c>
       <c r="D89" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E89" s="15" t="s">
-        <v>2718</v>
+        <v>2720</v>
       </c>
       <c r="F89" s="10" t="s">
         <v>63</v>
       </c>
       <c r="G89" s="9" t="s">
-        <v>2719</v>
+        <v>2721</v>
       </c>
       <c r="H89" s="10" t="s">
         <v>63</v>
@@ -54172,13 +54178,13 @@
     </row>
     <row r="90" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>2720</v>
+        <v>2722</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>2703</v>
+        <v>2705</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>2721</v>
+        <v>2723</v>
       </c>
       <c r="D90" s="10" t="s">
         <v>63</v>
@@ -54190,13 +54196,13 @@
         <v>63</v>
       </c>
       <c r="G90" s="15" t="s">
-        <v>2722</v>
+        <v>2724</v>
       </c>
       <c r="H90" s="15" t="s">
-        <v>2723</v>
+        <v>2725</v>
       </c>
       <c r="I90" s="15" t="s">
-        <v>2724</v>
+        <v>2726</v>
       </c>
       <c r="J90" s="2">
         <v>14</v>
@@ -54204,13 +54210,13 @@
     </row>
     <row r="91" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>2725</v>
+        <v>2727</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>2726</v>
+        <v>2728</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>2727</v>
+        <v>2729</v>
       </c>
       <c r="D91" s="10" t="s">
         <v>63</v>
@@ -54225,7 +54231,7 @@
         <v>63</v>
       </c>
       <c r="H91" s="15" t="s">
-        <v>2728</v>
+        <v>2730</v>
       </c>
       <c r="I91" s="10" t="s">
         <v>63</v>
@@ -54257,16 +54263,16 @@
         <v>32</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>2729</v>
+        <v>2731</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2730</v>
+        <v>2732</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>35</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>2731</v>
+        <v>2733</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -54274,16 +54280,16 @@
         <v>143</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>2732</v>
+        <v>2734</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>2733</v>
+        <v>2735</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>2734</v>
+        <v>2736</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>2735</v>
+        <v>2737</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -54291,16 +54297,16 @@
         <v>1340</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>2738</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>2739</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>2736</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>2737</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>2734</v>
-      </c>
       <c r="E3" s="2" t="s">
-        <v>2738</v>
+        <v>2740</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -54308,16 +54314,16 @@
         <v>110</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>2739</v>
+        <v>2741</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>2740</v>
+        <v>2742</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>2741</v>
+        <v>2743</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>2742</v>
+        <v>2744</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -54325,16 +54331,16 @@
         <v>920</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>2745</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>2746</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>2743</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>2744</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>2741</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>2735</v>
+        <v>2737</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -54342,16 +54348,16 @@
         <v>363</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>2745</v>
+        <v>2747</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>2746</v>
+        <v>2748</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>2734</v>
+        <v>2736</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>2735</v>
+        <v>2737</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -54359,16 +54365,16 @@
         <v>454</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>2747</v>
+        <v>2749</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>2748</v>
+        <v>2750</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>2734</v>
+        <v>2736</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>2735</v>
+        <v>2737</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -54376,16 +54382,16 @@
         <v>104</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>2749</v>
+        <v>2751</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>2750</v>
+        <v>2752</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>2734</v>
+        <v>2736</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>2751</v>
+        <v>2753</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -54393,33 +54399,33 @@
         <v>377</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>2752</v>
+        <v>2754</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>2753</v>
+        <v>2755</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>2734</v>
+        <v>2736</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>2735</v>
+        <v>2737</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>2754</v>
+        <v>2756</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>2755</v>
+        <v>2757</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>2756</v>
+        <v>2758</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>2734</v>
+        <v>2736</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>2735</v>
+        <v>2737</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -54427,59 +54433,59 @@
         <v>809</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>2757</v>
+        <v>2759</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>2758</v>
+        <v>2760</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>2759</v>
+        <v>2761</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>2760</v>
+        <v>2762</v>
       </c>
     </row>
     <row r="13" spans="2:2" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B13" s="17" t="s">
-        <v>2761</v>
+        <v>2763</v>
       </c>
     </row>
     <row r="14" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
-        <v>2762</v>
+        <v>2764</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>2763</v>
+        <v>2765</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>2764</v>
+        <v>2766</v>
       </c>
     </row>
     <row r="15" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
-        <v>2765</v>
+        <v>2767</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>2766</v>
+        <v>2768</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>2767</v>
+        <v>2769</v>
       </c>
     </row>
     <row r="16" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
-        <v>2768</v>
+        <v>2770</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>2769</v>
+        <v>2771</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>2770</v>
+        <v>2772</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>2771</v>
+        <v>2773</v>
       </c>
     </row>
   </sheetData>
@@ -54505,10 +54511,10 @@
         <v>33</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>2772</v>
+        <v>2774</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2773</v>
+        <v>2775</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>56</v>
@@ -54520,7 +54526,7 @@
         <v>64</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>2774</v>
+        <v>2776</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>102</v>
@@ -54540,7 +54546,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="B2" t="s">
         <v>51</v>
@@ -54578,7 +54584,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2646</v>
+        <v>2648</v>
       </c>
       <c r="B3" t="s">
         <v>397</v>
@@ -54616,7 +54622,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="B4" t="s">
         <v>541</v>
@@ -54654,7 +54660,7 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="B5" t="s">
         <v>702</v>
@@ -54692,7 +54698,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>2458</v>
+        <v>2460</v>
       </c>
       <c r="B6" t="s">
         <v>848</v>
@@ -54730,7 +54736,7 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="B7" t="s">
         <v>996</v>
@@ -54768,7 +54774,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>2573</v>
+        <v>2575</v>
       </c>
       <c r="B8" t="s">
         <v>1147</v>
@@ -54806,7 +54812,7 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>2545</v>
+        <v>2547</v>
       </c>
       <c r="B9" t="s">
         <v>1237</v>
@@ -54844,7 +54850,7 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>2586</v>
+        <v>2588</v>
       </c>
       <c r="B10" t="s">
         <v>1354</v>
@@ -54882,7 +54888,7 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>2597</v>
+        <v>2599</v>
       </c>
       <c r="B11" t="s">
         <v>1420</v>
@@ -54920,7 +54926,7 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>2617</v>
+        <v>2619</v>
       </c>
       <c r="B12" t="s">
         <v>1504</v>
@@ -54958,7 +54964,7 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>2635</v>
+        <v>2637</v>
       </c>
       <c r="B13" t="s">
         <v>1552</v>
@@ -54996,7 +55002,7 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>2689</v>
+        <v>2691</v>
       </c>
       <c r="B14" t="s">
         <v>1671</v>
@@ -55034,7 +55040,7 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>2622</v>
+        <v>2624</v>
       </c>
       <c r="B15" t="s">
         <v>1759</v>
@@ -55072,7 +55078,7 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>2703</v>
+        <v>2705</v>
       </c>
       <c r="B16" t="s">
         <v>1793</v>
@@ -55110,7 +55116,7 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>2775</v>
+        <v>2777</v>
       </c>
       <c r="B17" t="s">
         <v>1911</v>
@@ -55148,7 +55154,7 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>2726</v>
+        <v>2728</v>
       </c>
       <c r="B18" t="s">
         <v>1973</v>
@@ -55186,7 +55192,7 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>2776</v>
+        <v>2778</v>
       </c>
       <c r="B19" t="s">
         <v>2001</v>
@@ -55224,7 +55230,7 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>2709</v>
+        <v>2711</v>
       </c>
       <c r="B20" t="s">
         <v>2017</v>
@@ -55262,7 +55268,7 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>2777</v>
+        <v>2779</v>
       </c>
       <c r="B21" t="s">
         <v>2048</v>
@@ -55300,7 +55306,7 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>2778</v>
+        <v>2780</v>
       </c>
       <c r="B22" t="s">
         <v>2088</v>
@@ -55338,7 +55344,7 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>2779</v>
+        <v>2781</v>
       </c>
       <c r="B23" t="s">
         <v>2117</v>
@@ -55376,7 +55382,7 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>2780</v>
+        <v>2782</v>
       </c>
       <c r="B24" t="s">
         <v>2145</v>
@@ -55414,7 +55420,7 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>2781</v>
+        <v>2783</v>
       </c>
       <c r="B25" t="s">
         <v>2184</v>
@@ -55452,7 +55458,7 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>2782</v>
+        <v>2784</v>
       </c>
       <c r="B26" t="s">
         <v>2207</v>
@@ -55490,7 +55496,7 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>2783</v>
+        <v>2785</v>
       </c>
       <c r="B27" t="s">
         <v>2221</v>
@@ -55528,7 +55534,7 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>2784</v>
+        <v>2786</v>
       </c>
       <c r="B28" t="s">
         <v>2238</v>
@@ -55566,7 +55572,7 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>2785</v>
+        <v>2787</v>
       </c>
       <c r="B29" t="s">
         <v>2262</v>
@@ -55604,7 +55610,7 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>2786</v>
+        <v>2788</v>
       </c>
       <c r="B30" t="s">
         <v>2277</v>
@@ -55642,7 +55648,7 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>2787</v>
+        <v>2789</v>
       </c>
       <c r="B31" t="s">
         <v>2294</v>
@@ -55680,7 +55686,7 @@
     </row>
     <row r="33" spans="2:12" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B33" s="17" t="s">
-        <v>2773</v>
+        <v>2775</v>
       </c>
       <c r="C33" s="17">
         <v>559</v>

</xml_diff>

<commit_message>
docs: evidencia de recomendaciones explicadas (mejora M-08)
</commit_message>
<xml_diff>
--- a/docs/requisitos/FOOD4ALL_requisitos_benchmark.xlsx
+++ b/docs/requisitos/FOOD4ALL_requisitos_benchmark.xlsx
@@ -2392,10 +2392,10 @@
     <t>RF-04.5-04</t>
   </si>
   <si>
-    <t>Mostrar hasta 4 productos relacionados del mismo vendedor.</t>
-  </si>
-  <si>
-    <t>Dado un vendedor con 6 productos, cuando se abre uno, entonces se ven 4 relacionados.</t>
+    <t>Mostrar hasta 4 productos del mismo vendedor bajo el título «Más de &lt;vendedor&gt;», para que se vea el criterio.</t>
+  </si>
+  <si>
+    <t>Dado un vendedor con 6 productos, cuando se abre uno, entonces se ven 4 bajo «Más de &lt;vendedor&gt;».</t>
   </si>
   <si>
     <t xml:space="preserve">BF17 Perfil e historia del productor
@@ -4940,7 +4940,7 @@
     <t>BF68 Recomendaciones personalizadas</t>
   </si>
   <si>
-    <t>parcial en Glovo. Sin verificar: Too Good To Go, Wetaca, Market Wagon, Open Food Network.</t>
+    <t>Ningún competidor recorrido explica sus recomendaciones («Otros también compraron», «Productos relacionados», platos «similares»); solo la etiqueta ambiental de Open Food Network dice en qué se basa (recorrido del 23/10/2026). Datos: P: Glovo · N: Mercadona online · ?: Too Good To Go, Wetaca, Market Wagon, Open Food Network.</t>
   </si>
   <si>
     <t>RF-12.3-02</t>
@@ -36771,8 +36771,8 @@
       <c r="T373" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="U373" s="9" t="s">
-        <v>102</v>
+      <c r="U373" s="11" t="s">
+        <v>419</v>
       </c>
       <c r="V373" s="2" t="s">
         <v>1618</v>
@@ -55424,10 +55424,10 @@
         <v>0</v>
       </c>
       <c r="H13">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13">
         <v>2</v>
@@ -56140,10 +56140,10 @@
         <v>116</v>
       </c>
       <c r="H33" s="17">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="I33" s="17">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J33" s="17">
         <v>10</v>

</xml_diff>

<commit_message>
docs: criba B y D, entrevistas E5-E6, descarte de las de Miguel y RF-08.5-01 al MVP
</commit_message>
<xml_diff>
--- a/docs/requisitos/FOOD4ALL_requisitos_benchmark.xlsx
+++ b/docs/requisitos/FOOD4ALL_requisitos_benchmark.xlsx
@@ -4099,7 +4099,7 @@
     <t>Dado un lote retirado, cuando se confirma, entonces cada comprador recibe el aviso.</t>
   </si>
   <si>
-    <t>Comparado a nivel de función (Retirada y excedentes): parcial en Too Good To Go. Sin verificar: Mercadona online, Glovo, Wetaca, Market Wagon, Open Food Network.</t>
+    <t>Seguridad alimentaria (regla A.2 c de la criba): solo la plataforma sabe quién compró el lote, así que el aviso a los compradores es suyo sea cual sea D-01 (C-23). Datos: P: Too Good To Go · ?: Mercadona online, Glovo, Wetaca, Market Wagon, Open Food Network.</t>
   </si>
   <si>
     <t>RF-08.5-02</t>
@@ -31550,13 +31550,13 @@
         <v>1339</v>
       </c>
       <c r="G303" s="2" t="s">
-        <v>88</v>
+        <v>56</v>
       </c>
       <c r="H303" s="2" t="s">
-        <v>119</v>
+        <v>57</v>
       </c>
       <c r="I303" s="2" t="s">
-        <v>119</v>
+        <v>57</v>
       </c>
       <c r="J303" s="2" t="s">
         <v>1272</v>
@@ -51298,7 +51298,7 @@
         <v>37</v>
       </c>
       <c r="J9" s="2">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -55260,10 +55260,10 @@
         <v>29</v>
       </c>
       <c r="D9">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E9">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F9">
         <v>12</v>
@@ -56131,10 +56131,10 @@
         <v>564</v>
       </c>
       <c r="D33" s="17">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E33" s="17">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F33" s="17">
         <v>116</v>

</xml_diff>

<commit_message>
docs: E1-E6 coherentes en todos los documentos (C-25)
</commit_message>
<xml_diff>
--- a/docs/requisitos/FOOD4ALL_requisitos_benchmark.xlsx
+++ b/docs/requisitos/FOOD4ALL_requisitos_benchmark.xlsx
@@ -7106,7 +7106,7 @@
     <t>Indicio</t>
   </si>
   <si>
-    <t>F-01, F-02, F-07 (E3, E4)</t>
+    <t>F-01, F-02, F-07 (E3, E4, E6)</t>
   </si>
   <si>
     <t>N-01</t>
@@ -7115,7 +7115,7 @@
     <t>N-03, N-04, N-05</t>
   </si>
   <si>
-    <t>F-01, F-07 (E4; E1 comparativo)</t>
+    <t>F-01, F-07 (E4, E5, E6; E1 comparativo)</t>
   </si>
   <si>
     <t>F-04, F-10, F-07 (E4; E3 en contra del producto, no de la necesidad)</t>
@@ -7127,13 +7127,13 @@
     <t>N-02, N-08</t>
   </si>
   <si>
-    <t>F-04, F-05</t>
+    <t>F-04, F-07 (solo E1, comparativo: entrega en 1–4 días)</t>
   </si>
   <si>
     <t>N-10</t>
   </si>
   <si>
-    <t>F-01, F-03, F-07 (E3, E4)</t>
+    <t>F-01, F-03, F-07 (E3; en contra: E4)</t>
   </si>
   <si>
     <t>N-08</t>
@@ -7166,7 +7166,7 @@
     <t>—</t>
   </si>
   <si>
-    <t>F-03 (Reglamento 178/2002), F-04, F-07 (E4; E1 y E2 comparativos)</t>
+    <t>F-03 (Reglamento 178/2002), F-04, F-07 (E4; E5 y E6 comprueban la fiabilidad de una app antes de usarla; en contra del origen: E6; E1 y E2 comparativos)</t>
   </si>
   <si>
     <t>N-04 y N-05 (parte)</t>
@@ -7190,7 +7190,7 @@
     <t>F-03 (RGPD; LOPDGDD)</t>
   </si>
   <si>
-    <t>F-04 (fiabilidad baja: no cita fuentes)</t>
+    <t>F-04 (fiabilidad baja: no cita fuentes), F-07 (E5)</t>
   </si>
   <si>
     <t>N-06</t>
@@ -51414,7 +51414,7 @@
         <v>2334</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>922</v>
+        <v>2335</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>2364</v>

</xml_diff>